<commit_message>
Add the five councils covering the listed sites to the Outreach tab
Whittlesea, Mitchell, Wyndham, Melton and Greater Geelong each get a row
with their published general inbox, phone and contact page, and a message
addressed to the property and strategic acquisitions team that names the
sites in that council's area first.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Developer List'!$A$1:$V$197</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Outreach'!$A$1:$N$175</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Outreach'!$A$1:$N$180</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cross-check'!$A$1:$B$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'UDIA All Members'!$A$1:$H$386</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sources &amp; Notes'!$A$1:$B$11</definedName>
@@ -16142,7 +16142,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N199"/>
+  <dimension ref="A1:N204"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -16164,7 +16164,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Developer</t>
+          <t>Developer / council</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -29415,137 +29415,482 @@
       <c r="M175" s="2" t="inlineStr"/>
       <c r="N175" s="2" t="inlineStr"/>
     </row>
-    <row r="177">
-      <c r="A177" s="6" t="inlineStr">
+    <row r="176" ht="150" customHeight="1">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>City of Whittlesea</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>https://www.whittlesea.vic.gov.au/About-us/Contact-us</t>
+        </is>
+      </c>
+      <c r="C176" s="4" t="inlineStr">
+        <is>
+          <t>https://www.whittlesea.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>info@whittlesea.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="E176" s="2" t="inlineStr">
+        <is>
+          <t>03 9217 2170</t>
+        </is>
+      </c>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>Inder Sandhu</t>
+        </is>
+      </c>
+      <c r="G176" s="2" t="inlineStr">
+        <is>
+          <t>inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="H176" s="2" t="inlineStr">
+        <is>
+          <t>0484926324</t>
+        </is>
+      </c>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="J176" s="2" t="inlineStr">
+        <is>
+          <t>Development sites in Wollert</t>
+        </is>
+      </c>
+      <c r="K176" s="3" t="inlineStr">
+        <is>
+          <t>Hi Property and Strategic Acquisitions Team,
+My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
+I have development sites available in Wollert, within the City of Whittlesea's area, as well as in Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+* Shovel-ready residential and industrial.
+* Permit-approved townhouse sites, including one for 44 townhouses.
+* Childcare and townhouse sites, both raw and approved.
+* About 50 acres of investigation-area land.
+Given Council's role in planning for growth in Wollert, some of these sites may suit Council's strategic land or community infrastructure needs.
+Could you please forward this to the appropriate contact in Council's property or strategic acquisitions team so I can share further details?
+If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Kind regards,
+Inder Sandhu
+Crown Real Estate Agents
+0484 926 324 | inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="L176" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="M176" s="2" t="inlineStr"/>
+      <c r="N176" s="2" t="inlineStr">
+        <is>
+          <t>Local council – sites in Wollert. General inbox; email source: council annual report 2022-23 and official Facebook page</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="150" customHeight="1">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>Mitchell Shire Council</t>
+        </is>
+      </c>
+      <c r="B177" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mitchellshire.vic.gov.au/contact</t>
+        </is>
+      </c>
+      <c r="C177" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mitchellshire.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>mitchell@mitchellshire.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="E177" s="2" t="inlineStr">
+        <is>
+          <t>03 5734 6200</t>
+        </is>
+      </c>
+      <c r="F177" s="2" t="inlineStr">
+        <is>
+          <t>Inder Sandhu</t>
+        </is>
+      </c>
+      <c r="G177" s="2" t="inlineStr">
+        <is>
+          <t>inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="H177" s="2" t="inlineStr">
+        <is>
+          <t>0484926324</t>
+        </is>
+      </c>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="J177" s="2" t="inlineStr">
+        <is>
+          <t>Development sites in Beveridge</t>
+        </is>
+      </c>
+      <c r="K177" s="3" t="inlineStr">
+        <is>
+          <t>Hi Property and Strategic Acquisitions Team,
+My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
+I have development sites available in Beveridge, within Mitchell Shire Council's area, as well as in Wollert, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+* Shovel-ready residential and industrial.
+* Permit-approved townhouse sites, including one for 44 townhouses.
+* Childcare and townhouse sites, both raw and approved.
+* About 50 acres of investigation-area land.
+Given Council's role in planning for growth in Beveridge, some of these sites may suit Council's strategic land or community infrastructure needs.
+Could you please forward this to the appropriate contact in Council's property or strategic acquisitions team so I can share further details?
+If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Kind regards,
+Inder Sandhu
+Crown Real Estate Agents
+0484 926 324 | inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="L177" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="M177" s="2" t="inlineStr"/>
+      <c r="N177" s="2" t="inlineStr">
+        <is>
+          <t>Local council – sites in Beveridge. General inbox; email source: council contact page</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="150" customHeight="1">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>Wyndham City Council</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wyndham.vic.gov.au/contact-us</t>
+        </is>
+      </c>
+      <c r="C178" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wyndham.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>mail@wyndham.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="E178" s="2" t="inlineStr">
+        <is>
+          <t>1300 023 411</t>
+        </is>
+      </c>
+      <c r="F178" s="2" t="inlineStr">
+        <is>
+          <t>Inder Sandhu</t>
+        </is>
+      </c>
+      <c r="G178" s="2" t="inlineStr">
+        <is>
+          <t>inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="H178" s="2" t="inlineStr">
+        <is>
+          <t>0484926324</t>
+        </is>
+      </c>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="J178" s="2" t="inlineStr">
+        <is>
+          <t>Development sites in Tarneit &amp; Truganina</t>
+        </is>
+      </c>
+      <c r="K178" s="3" t="inlineStr">
+        <is>
+          <t>Hi Property and Strategic Acquisitions Team,
+My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
+I have development sites available in Tarneit and Truganina, within Wyndham City Council's area, as well as in Wollert, Beveridge, Geelong, Deanside, Bonnie Brook and Fraser Rise:
+* Shovel-ready residential and industrial.
+* Permit-approved townhouse sites, including one for 44 townhouses.
+* Childcare and townhouse sites, both raw and approved.
+* About 50 acres of investigation-area land.
+Given Council's role in planning for growth in Tarneit and Truganina, some of these sites may suit Council's strategic land or community infrastructure needs.
+Could you please forward this to the appropriate contact in Council's property or strategic acquisitions team so I can share further details?
+If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Kind regards,
+Inder Sandhu
+Crown Real Estate Agents
+0484 926 324 | inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="L178" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="M178" s="2" t="inlineStr"/>
+      <c r="N178" s="2" t="inlineStr">
+        <is>
+          <t>Local council – sites in Tarneit and Truganina. General inbox; email source: council contact page</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="150" customHeight="1">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>Melton City Council</t>
+        </is>
+      </c>
+      <c r="B179" s="4" t="inlineStr">
+        <is>
+          <t>https://www.melton.vic.gov.au/Council/Customer-Service/Contact-Us</t>
+        </is>
+      </c>
+      <c r="C179" s="4" t="inlineStr">
+        <is>
+          <t>https://www.melton.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>csu@melton.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="E179" s="2" t="inlineStr">
+        <is>
+          <t>03 9747 7200</t>
+        </is>
+      </c>
+      <c r="F179" s="2" t="inlineStr">
+        <is>
+          <t>Inder Sandhu</t>
+        </is>
+      </c>
+      <c r="G179" s="2" t="inlineStr">
+        <is>
+          <t>inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="H179" s="2" t="inlineStr">
+        <is>
+          <t>0484926324</t>
+        </is>
+      </c>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="J179" s="2" t="inlineStr">
+        <is>
+          <t>Development sites in Deanside, Bonnie Brook &amp; Fraser Rise</t>
+        </is>
+      </c>
+      <c r="K179" s="3" t="inlineStr">
+        <is>
+          <t>Hi Property and Strategic Acquisitions Team,
+My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
+I have development sites available in Deanside, Bonnie Brook and Fraser Rise, within Melton City Council's area, as well as in Wollert, Beveridge, Tarneit, Geelong and Truganina:
+* Shovel-ready residential and industrial.
+* Permit-approved townhouse sites, including one for 44 townhouses.
+* Childcare and townhouse sites, both raw and approved.
+* About 50 acres of investigation-area land.
+Given Council's role in planning for growth in Deanside, Bonnie Brook and Fraser Rise, some of these sites may suit Council's strategic land or community infrastructure needs.
+Could you please forward this to the appropriate contact in Council's property or strategic acquisitions team so I can share further details?
+If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Kind regards,
+Inder Sandhu
+Crown Real Estate Agents
+0484 926 324 | inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="L179" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="M179" s="2" t="inlineStr"/>
+      <c r="N179" s="2" t="inlineStr">
+        <is>
+          <t>Local council – sites in Deanside, Bonnie Brook and Fraser Rise. General inbox; email source: business.gov.au and vic.gov.au council listings</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="150" customHeight="1">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>City of Greater Geelong</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>https://www.geelongcity.vic.gov.au/contact</t>
+        </is>
+      </c>
+      <c r="C180" s="4" t="inlineStr">
+        <is>
+          <t>https://www.geelongcity.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>contactus@geelongcity.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="E180" s="2" t="inlineStr">
+        <is>
+          <t>03 5272 5272</t>
+        </is>
+      </c>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>Inder Sandhu</t>
+        </is>
+      </c>
+      <c r="G180" s="2" t="inlineStr">
+        <is>
+          <t>inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="H180" s="2" t="inlineStr">
+        <is>
+          <t>0484926324</t>
+        </is>
+      </c>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="J180" s="2" t="inlineStr">
+        <is>
+          <t>Development sites in Geelong</t>
+        </is>
+      </c>
+      <c r="K180" s="3" t="inlineStr">
+        <is>
+          <t>Hi Property and Strategic Acquisitions Team,
+My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
+I have development sites available in Geelong, within the City of Greater Geelong's area, as well as in Wollert, Beveridge, Tarneit, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+* Shovel-ready residential and industrial.
+* Permit-approved townhouse sites, including one for 44 townhouses.
+* Childcare and townhouse sites, both raw and approved.
+* About 50 acres of investigation-area land.
+Given Council's role in planning for growth in Geelong, some of these sites may suit Council's strategic land or community infrastructure needs.
+Could you please forward this to the appropriate contact in Council's property or strategic acquisitions team so I can share further details?
+If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Kind regards,
+Inder Sandhu
+Crown Real Estate Agents
+0484 926 324 | inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="L180" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="M180" s="2" t="inlineStr"/>
+      <c r="N180" s="2" t="inlineStr">
+        <is>
+          <t>Local council – sites in Geelong. General inbox; email source: council customer service charter and business.gov.au</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="6" t="inlineStr">
         <is>
           <t>Left out of outreach (and why):</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="7" t="inlineStr">
-        <is>
-          <t>Antipodean Land Developments</t>
-        </is>
-      </c>
-      <c r="B178" s="7" t="inlineStr">
-        <is>
-          <t>Only contact is a personal gmail</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="7" t="inlineStr">
-        <is>
-          <t>AVJennings</t>
-        </is>
-      </c>
-      <c r="B179" s="7" t="inlineStr">
-        <is>
-          <t>Website now redirects to AVID Property Group — contact AVID instead</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="7" t="inlineStr">
-        <is>
-          <t>Banner Asset Management</t>
-        </is>
-      </c>
-      <c r="B180" s="7" t="inlineStr">
-        <is>
-          <t>Finance firm</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="7" t="inlineStr">
-        <is>
-          <t>Bolton Clarke</t>
-        </is>
-      </c>
-      <c r="B181" s="7" t="inlineStr">
-        <is>
-          <t>Aged-care not-for-profit</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="7" t="inlineStr">
-        <is>
-          <t>Cambrooke Property Pty Ltd</t>
-        </is>
-      </c>
-      <c r="B182" s="7" t="inlineStr">
-        <is>
-          <t>Only selling-agent contact</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="7" t="inlineStr">
         <is>
-          <t>Community Housing Victoria Ltd</t>
+          <t>Antipodean Land Developments</t>
         </is>
       </c>
       <c r="B183" s="7" t="inlineStr">
         <is>
-          <t>Community housing provider</t>
+          <t>Only contact is a personal gmail</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="7" t="inlineStr">
         <is>
-          <t>Development Victoria</t>
+          <t>AVJennings</t>
         </is>
       </c>
       <c r="B184" s="7" t="inlineStr">
         <is>
-          <t>Government agency</t>
+          <t>Website now redirects to AVID Property Group — contact AVID instead</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="7" t="inlineStr">
         <is>
-          <t>Eight Property Investments</t>
+          <t>Banner Asset Management</t>
         </is>
       </c>
       <c r="B185" s="7" t="inlineStr">
         <is>
-          <t>In liquidation (ASIC notice)</t>
+          <t>Finance firm</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="7" t="inlineStr">
         <is>
-          <t>Homes Victoria</t>
+          <t>Bolton Clarke</t>
         </is>
       </c>
       <c r="B186" s="7" t="inlineStr">
         <is>
-          <t>Government agency</t>
+          <t>Aged-care not-for-profit</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="7" t="inlineStr">
         <is>
-          <t>Housing Choices Australia Limited (Victoria)</t>
+          <t>Cambrooke Property Pty Ltd</t>
         </is>
       </c>
       <c r="B187" s="7" t="inlineStr">
         <is>
-          <t>Community housing provider</t>
+          <t>Only selling-agent contact</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="7" t="inlineStr">
         <is>
-          <t>HousingFirst Ltd</t>
+          <t>Community Housing Victoria Ltd</t>
         </is>
       </c>
       <c r="B188" s="7" t="inlineStr">
@@ -29557,67 +29902,67 @@
     <row r="189">
       <c r="A189" s="7" t="inlineStr">
         <is>
-          <t>Hunter Park Country Estate developer (entity not identified)</t>
+          <t>Development Victoria</t>
         </is>
       </c>
       <c r="B189" s="7" t="inlineStr">
         <is>
-          <t>Developer not identified; only agent contact</t>
+          <t>Government agency</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="7" t="inlineStr">
         <is>
-          <t>Launch Housing</t>
+          <t>Eight Property Investments</t>
         </is>
       </c>
       <c r="B190" s="7" t="inlineStr">
         <is>
-          <t>Homelessness charity</t>
+          <t>In liquidation (ASIC notice)</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="7" t="inlineStr">
         <is>
-          <t>LOGOS</t>
+          <t>Homes Victoria</t>
         </is>
       </c>
       <c r="B191" s="7" t="inlineStr">
         <is>
-          <t>Site now redirects to ESR Australia — contact ESR instead</t>
+          <t>Government agency</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="7" t="inlineStr">
         <is>
-          <t>Montego Homes</t>
+          <t>Housing Choices Australia Limited (Victoria)</t>
         </is>
       </c>
       <c r="B192" s="7" t="inlineStr">
         <is>
-          <t>Collapsed in 2024</t>
+          <t>Community housing provider</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="7" t="inlineStr">
         <is>
-          <t>Mount Atkinson Holdings</t>
+          <t>HousingFirst Ltd</t>
         </is>
       </c>
       <c r="B193" s="7" t="inlineStr">
         <is>
-          <t>Domain no longer belongs to the company</t>
+          <t>Community housing provider</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="7" t="inlineStr">
         <is>
-          <t>Narracan Meadows developer (entity not identified)</t>
+          <t>Hunter Park Country Estate developer (entity not identified)</t>
         </is>
       </c>
       <c r="B194" s="7" t="inlineStr">
@@ -29629,65 +29974,125 @@
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
         <is>
-          <t>Seebeck Group Enterprise</t>
+          <t>Launch Housing</t>
         </is>
       </c>
       <c r="B195" s="7" t="inlineStr">
         <is>
-          <t>No contact details</t>
+          <t>Homelessness charity</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
         <is>
-          <t>Sunrise Ventures</t>
+          <t>LOGOS</t>
         </is>
       </c>
       <c r="B196" s="7" t="inlineStr">
         <is>
-          <t>No public contact details</t>
+          <t>Site now redirects to ESR Australia — contact ESR instead</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
         <is>
-          <t>The Range (Trafalgar) Pty Ltd</t>
+          <t>Montego Homes</t>
         </is>
       </c>
       <c r="B197" s="7" t="inlineStr">
         <is>
-          <t>Landowner entity, no contacts</t>
+          <t>Collapsed in 2024</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
         <is>
-          <t>Three Thirds Group</t>
+          <t>Mount Atkinson Holdings</t>
         </is>
       </c>
       <c r="B198" s="7" t="inlineStr">
         <is>
-          <t>Professional services firm</t>
+          <t>Domain no longer belongs to the company</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
         <is>
+          <t>Narracan Meadows developer (entity not identified)</t>
+        </is>
+      </c>
+      <c r="B199" s="7" t="inlineStr">
+        <is>
+          <t>Developer not identified; only agent contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="7" t="inlineStr">
+        <is>
+          <t>Seebeck Group Enterprise</t>
+        </is>
+      </c>
+      <c r="B200" s="7" t="inlineStr">
+        <is>
+          <t>No contact details</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="7" t="inlineStr">
+        <is>
+          <t>Sunrise Ventures</t>
+        </is>
+      </c>
+      <c r="B201" s="7" t="inlineStr">
+        <is>
+          <t>No public contact details</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="7" t="inlineStr">
+        <is>
+          <t>The Range (Trafalgar) Pty Ltd</t>
+        </is>
+      </c>
+      <c r="B202" s="7" t="inlineStr">
+        <is>
+          <t>Landowner entity, no contacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="7" t="inlineStr">
+        <is>
+          <t>Three Thirds Group</t>
+        </is>
+      </c>
+      <c r="B203" s="7" t="inlineStr">
+        <is>
+          <t>Professional services firm</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="7" t="inlineStr">
+        <is>
           <t>Trafalgar Property Developments Pty Ltd</t>
         </is>
       </c>
-      <c r="B199" s="7" t="inlineStr">
+      <c r="B204" s="7" t="inlineStr">
         <is>
           <t>Landowner entity, no contacts</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N175"/>
+  <autoFilter ref="A1:N180"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId2"/>
@@ -30020,6 +30425,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C174" r:id="rId329"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B175" r:id="rId330"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C175" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B176" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C176" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B177" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C177" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B178" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C178" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B179" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C179" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B180" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C180" r:id="rId341"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add the Bendigo, Ballarat, Shepparton and Latrobe councils to the Outreach tab
None of the listed sites sit in these four councils' areas, so their message
asks about Council's strategic land priorities rather than offering a local
site, and names the current sites only as examples.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Developer List'!$A$1:$V$197</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Outreach'!$A$1:$N$188</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Outreach'!$A$1:$N$192</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cross-check'!$A$1:$B$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'UDIA All Members'!$A$1:$H$386</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sources &amp; Notes'!$A$1:$B$11</definedName>
@@ -16177,7 +16177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N204"/>
+  <dimension ref="A1:N208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -30451,125 +30451,401 @@
         </is>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="6" t="inlineStr">
+    <row r="189" ht="150" customHeight="1">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>City of Greater Bendigo</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bendigo.vic.gov.au/contact-us</t>
+        </is>
+      </c>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bendigo.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>requests@bendigo.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="E189" s="2" t="inlineStr">
+        <is>
+          <t>1300 002 642</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>Inder Sandhu</t>
+        </is>
+      </c>
+      <c r="G189" s="2" t="inlineStr">
+        <is>
+          <t>inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="H189" s="2" t="inlineStr">
+        <is>
+          <t>0484926324</t>
+        </is>
+      </c>
+      <c r="I189" s="2" t="inlineStr">
+        <is>
+          <t>Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="J189" s="2" t="inlineStr">
+        <is>
+          <t>Development land – Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="K189" s="3" t="inlineStr">
+        <is>
+          <t>Hi Property and Strategic Acquisitions Team,
+My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria, including Greater Bendigo.
+I currently have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+* Shovel-ready residential and industrial.
+* Permit-approved townhouse sites, including one for 44 townhouses.
+* Childcare and townhouse sites, both raw and approved.
+* About 50 acres of investigation-area land.
+Given Council's role in planning for growth in Greater Bendigo, I'd welcome the chance to understand Council's strategic land priorities, so I can bring you suitable sites as they come up.
+Could you please forward this to the appropriate contact in Council's property or strategic acquisitions team?
+If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Kind regards,
+Inder Sandhu
+Crown Real Estate Agents
+0484 926 324 | inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="L189" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="M189" s="2" t="inlineStr"/>
+      <c r="N189" s="2" t="inlineStr">
+        <is>
+          <t>Regional council – no listed site in its area yet. General inbox; email source: council contact page</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="150" customHeight="1">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>City of Ballarat</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ballarat.vic.gov.au/about-us/contact-us</t>
+        </is>
+      </c>
+      <c r="C190" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ballarat.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>info@ballarat.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>03 5320 5500</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="inlineStr">
+        <is>
+          <t>Inder Sandhu</t>
+        </is>
+      </c>
+      <c r="G190" s="2" t="inlineStr">
+        <is>
+          <t>inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="H190" s="2" t="inlineStr">
+        <is>
+          <t>0484926324</t>
+        </is>
+      </c>
+      <c r="I190" s="2" t="inlineStr">
+        <is>
+          <t>Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="J190" s="2" t="inlineStr">
+        <is>
+          <t>Development land – Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="K190" s="3" t="inlineStr">
+        <is>
+          <t>Hi Property and Strategic Acquisitions Team,
+My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria, including Ballarat.
+I currently have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+* Shovel-ready residential and industrial.
+* Permit-approved townhouse sites, including one for 44 townhouses.
+* Childcare and townhouse sites, both raw and approved.
+* About 50 acres of investigation-area land.
+Given Council's role in planning for growth in Ballarat, I'd welcome the chance to understand Council's strategic land priorities, so I can bring you suitable sites as they come up.
+Could you please forward this to the appropriate contact in Council's property or strategic acquisitions team?
+If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Kind regards,
+Inder Sandhu
+Crown Real Estate Agents
+0484 926 324 | inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="L190" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="M190" s="2" t="inlineStr"/>
+      <c r="N190" s="2" t="inlineStr">
+        <is>
+          <t>Regional council – no listed site in its area yet. General inbox; email source: council contact page (phone from council eServices page)</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="150" customHeight="1">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>Greater Shepparton City Council</t>
+        </is>
+      </c>
+      <c r="B191" s="4" t="inlineStr">
+        <is>
+          <t>https://greatershepparton.com.au/</t>
+        </is>
+      </c>
+      <c r="C191" s="4" t="inlineStr">
+        <is>
+          <t>https://greatershepparton.com.au</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>council@shepparton.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="E191" s="2" t="inlineStr">
+        <is>
+          <t>03 5832 9700</t>
+        </is>
+      </c>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>Inder Sandhu</t>
+        </is>
+      </c>
+      <c r="G191" s="2" t="inlineStr">
+        <is>
+          <t>inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="H191" s="2" t="inlineStr">
+        <is>
+          <t>0484926324</t>
+        </is>
+      </c>
+      <c r="I191" s="2" t="inlineStr">
+        <is>
+          <t>Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="J191" s="2" t="inlineStr">
+        <is>
+          <t>Development land – Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="K191" s="3" t="inlineStr">
+        <is>
+          <t>Hi Property and Strategic Acquisitions Team,
+My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria, including Greater Shepparton.
+I currently have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+* Shovel-ready residential and industrial.
+* Permit-approved townhouse sites, including one for 44 townhouses.
+* Childcare and townhouse sites, both raw and approved.
+* About 50 acres of investigation-area land.
+Given Council's role in planning for growth in Greater Shepparton, I'd welcome the chance to understand Council's strategic land priorities, so I can bring you suitable sites as they come up.
+Could you please forward this to the appropriate contact in Council's property or strategic acquisitions team?
+If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Kind regards,
+Inder Sandhu
+Crown Real Estate Agents
+0484 926 324 | inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="L191" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="M191" s="2" t="inlineStr"/>
+      <c r="N191" s="2" t="inlineStr">
+        <is>
+          <t>Regional council – no listed site in its area yet. General inbox; email source: business.gov.au and OVIC agency listings</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="150" customHeight="1">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Latrobe City Council</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>https://www.latrobe.vic.gov.au/Contact_Us</t>
+        </is>
+      </c>
+      <c r="C192" s="4" t="inlineStr">
+        <is>
+          <t>https://www.latrobe.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>latrobe@latrobe.vic.gov.au</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>1300 367 700</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="inlineStr">
+        <is>
+          <t>Inder Sandhu</t>
+        </is>
+      </c>
+      <c r="G192" s="2" t="inlineStr">
+        <is>
+          <t>inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="H192" s="2" t="inlineStr">
+        <is>
+          <t>0484926324</t>
+        </is>
+      </c>
+      <c r="I192" s="2" t="inlineStr">
+        <is>
+          <t>Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="J192" s="2" t="inlineStr">
+        <is>
+          <t>Development land – Crown Real Estate Agents</t>
+        </is>
+      </c>
+      <c r="K192" s="3" t="inlineStr">
+        <is>
+          <t>Hi Property and Strategic Acquisitions Team,
+My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria, including Latrobe, including Moe and Newborough.
+I currently have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+* Shovel-ready residential and industrial.
+* Permit-approved townhouse sites, including one for 44 townhouses.
+* Childcare and townhouse sites, both raw and approved.
+* About 50 acres of investigation-area land.
+Given Council's role in planning for growth in Latrobe, including Moe and Newborough, I'd welcome the chance to understand Council's strategic land priorities, so I can bring you suitable sites as they come up.
+Could you please forward this to the appropriate contact in Council's property or strategic acquisitions team?
+If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Kind regards,
+Inder Sandhu
+Crown Real Estate Agents
+0484 926 324 | inder@crownrea.com.au</t>
+        </is>
+      </c>
+      <c r="L192" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="M192" s="2" t="inlineStr"/>
+      <c r="N192" s="2" t="inlineStr">
+        <is>
+          <t>Regional council – no listed site in its area yet. General inbox; email source: council contact page and vic.gov.au listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="6" t="inlineStr">
         <is>
           <t>Left out of outreach (and why):</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" s="7" t="inlineStr">
-        <is>
-          <t>Antipodean Land Developments</t>
-        </is>
-      </c>
-      <c r="B191" s="7" t="inlineStr">
-        <is>
-          <t>Only contact is a personal gmail</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="7" t="inlineStr">
-        <is>
-          <t>AVJennings</t>
-        </is>
-      </c>
-      <c r="B192" s="7" t="inlineStr">
-        <is>
-          <t>Website now redirects to AVID Property Group — contact AVID instead</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="7" t="inlineStr">
-        <is>
-          <t>Banner Asset Management</t>
-        </is>
-      </c>
-      <c r="B193" s="7" t="inlineStr">
-        <is>
-          <t>Finance firm</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" s="7" t="inlineStr">
-        <is>
-          <t>Cambrooke Property Pty Ltd</t>
-        </is>
-      </c>
-      <c r="B194" s="7" t="inlineStr">
-        <is>
-          <t>Only selling-agent contact</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="7" t="inlineStr">
         <is>
-          <t>Eight Property Investments</t>
+          <t>Antipodean Land Developments</t>
         </is>
       </c>
       <c r="B195" s="7" t="inlineStr">
         <is>
-          <t>In liquidation (ASIC notice)</t>
+          <t>Only contact is a personal gmail</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="7" t="inlineStr">
         <is>
-          <t>Hunter Park Country Estate developer (entity not identified)</t>
+          <t>AVJennings</t>
         </is>
       </c>
       <c r="B196" s="7" t="inlineStr">
         <is>
-          <t>Developer not identified; only agent contact</t>
+          <t>Website now redirects to AVID Property Group — contact AVID instead</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="7" t="inlineStr">
         <is>
-          <t>LOGOS</t>
+          <t>Banner Asset Management</t>
         </is>
       </c>
       <c r="B197" s="7" t="inlineStr">
         <is>
-          <t>Site now redirects to ESR Australia — contact ESR instead</t>
+          <t>Finance firm</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="7" t="inlineStr">
         <is>
-          <t>Montego Homes</t>
+          <t>Cambrooke Property Pty Ltd</t>
         </is>
       </c>
       <c r="B198" s="7" t="inlineStr">
         <is>
-          <t>Collapsed in 2024</t>
+          <t>Only selling-agent contact</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="7" t="inlineStr">
         <is>
-          <t>Mount Atkinson Holdings</t>
+          <t>Eight Property Investments</t>
         </is>
       </c>
       <c r="B199" s="7" t="inlineStr">
         <is>
-          <t>Domain no longer belongs to the company</t>
+          <t>In liquidation (ASIC notice)</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="7" t="inlineStr">
         <is>
-          <t>Narracan Meadows developer (entity not identified)</t>
+          <t>Hunter Park Country Estate developer (entity not identified)</t>
         </is>
       </c>
       <c r="B200" s="7" t="inlineStr">
@@ -30581,53 +30857,101 @@
     <row r="201">
       <c r="A201" s="7" t="inlineStr">
         <is>
-          <t>Sunrise Ventures</t>
+          <t>LOGOS</t>
         </is>
       </c>
       <c r="B201" s="7" t="inlineStr">
         <is>
-          <t>No public contact details</t>
+          <t>Site now redirects to ESR Australia — contact ESR instead</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="7" t="inlineStr">
         <is>
-          <t>The Range (Trafalgar) Pty Ltd</t>
+          <t>Montego Homes</t>
         </is>
       </c>
       <c r="B202" s="7" t="inlineStr">
         <is>
-          <t>Landowner entity, no contacts</t>
+          <t>Collapsed in 2024</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="7" t="inlineStr">
         <is>
-          <t>Three Thirds Group</t>
+          <t>Mount Atkinson Holdings</t>
         </is>
       </c>
       <c r="B203" s="7" t="inlineStr">
         <is>
-          <t>Professional services firm</t>
+          <t>Domain no longer belongs to the company</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="7" t="inlineStr">
         <is>
+          <t>Narracan Meadows developer (entity not identified)</t>
+        </is>
+      </c>
+      <c r="B204" s="7" t="inlineStr">
+        <is>
+          <t>Developer not identified; only agent contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="7" t="inlineStr">
+        <is>
+          <t>Sunrise Ventures</t>
+        </is>
+      </c>
+      <c r="B205" s="7" t="inlineStr">
+        <is>
+          <t>No public contact details</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="7" t="inlineStr">
+        <is>
+          <t>The Range (Trafalgar) Pty Ltd</t>
+        </is>
+      </c>
+      <c r="B206" s="7" t="inlineStr">
+        <is>
+          <t>Landowner entity, no contacts</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="7" t="inlineStr">
+        <is>
+          <t>Three Thirds Group</t>
+        </is>
+      </c>
+      <c r="B207" s="7" t="inlineStr">
+        <is>
+          <t>Professional services firm</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="7" t="inlineStr">
+        <is>
           <t>Trafalgar Property Developments Pty Ltd</t>
         </is>
       </c>
-      <c r="B204" s="7" t="inlineStr">
+      <c r="B208" s="7" t="inlineStr">
         <is>
           <t>Landowner entity, no contacts</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N188"/>
+  <autoFilter ref="A1:N192"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId2"/>
@@ -30985,6 +31309,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C187" r:id="rId354"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B188" r:id="rId355"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C188" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B189" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C189" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B190" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C190" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B191" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C191" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B192" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C192" r:id="rId364"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Use the shorter "Quick one" message on the Outreach tab
Developer and not-for-profit rows now carry the short message the user
chose, naming one of the developer's own projects ("especially alongside
Mandalay in Beveridge") where the data has one, and dropping that clause
where it doesn't. Councils keep their council-specific messages.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -16321,16 +16321,14 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit 3L Alliance's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given 3L Alliance's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -16406,16 +16404,14 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Abiwood's pipeline, especially alongside Pinnacle Ballarat in Smythes Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Abiwood's active presence in Ballarat, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -16487,16 +16483,14 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit ABN Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given ABN Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -16572,16 +16566,14 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Accord Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Accord Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -16653,16 +16645,14 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Mirrastone's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Mirrastone's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -16738,16 +16728,14 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Aliro Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Aliro Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -16823,16 +16811,14 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Allam Property Group's pipeline, especially alongside Alkyra in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Allam Property Group's active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -16904,16 +16890,14 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Anthela GPH Developments' pipeline, especially alongside Evermore in Kilmore:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Anthela GPH Developments' active presence in Kilmore, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -16981,16 +16965,14 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Antipodean Land Developments' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Antipodean Land Developments' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17066,16 +17048,14 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit APD Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given APD Projects' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17151,16 +17131,14 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Arc Living's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Arc Living's active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17236,16 +17214,14 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Assemble Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Assemble Communities' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17321,16 +17297,14 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit AVID Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given AVID Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17406,16 +17380,14 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Balcon Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Balcon Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17487,16 +17459,14 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bamfa Properties' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Bamfa Properties' active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17572,16 +17542,14 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Banco Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Banco Management's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17653,16 +17621,14 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Banner Asset Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Banner Asset Management's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17738,16 +17704,14 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Barks 33's pipeline, especially alongside Forest Ridge in Strathfieldsaye:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Barks 33's active presence in Bendigo, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17823,16 +17787,14 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bauenort's pipeline, especially alongside Alto Ballarat in Winter Valley:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Bauenort's active presence in Ballarat, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17904,16 +17866,14 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bayport's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Bayport's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -17985,16 +17945,14 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Begley Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Begley Group's active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18062,16 +18020,14 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bennett Williams' pipeline, especially alongside Heritage Estate in Moe:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Bennett Williams' active presence in Moe, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18143,16 +18099,14 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Beulah's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Beulah's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18228,16 +18182,14 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bevan Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Bevan Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18313,16 +18265,14 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Birchgrove Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Birchgrove Property's active presence in Bendigo, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18398,16 +18348,14 @@
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bisinella Developments' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Bisinella Developments' active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18483,16 +18431,14 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit BMD Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given BMD Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18564,16 +18510,14 @@
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bolton Clarke's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Bolton Clarke's role in delivering retirement living and aged care communities across Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18645,16 +18589,14 @@
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Brennan Development Group's pipeline, especially alongside Golden Grove Bendigo in Jackass Flat:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Brennan Development Group's active presence in Bendigo, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18730,16 +18672,14 @@
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Brown Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Brown Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18811,16 +18751,14 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Buildcap Development Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Buildcap Development Management's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18896,16 +18834,14 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Burbank Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Burbank Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -18977,16 +18913,14 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Cadence Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Cadence Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19062,16 +18996,14 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Carlisle Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Carlisle Homes' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19147,16 +19079,14 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Cedar Woods' pipeline, especially alongside Somerley in Corio:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Cedar Woods' active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19232,16 +19162,14 @@
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Central Equity's pipeline, especially alongside Palomino in Armstrong Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Central Equity's active presence in Geelong and Armstrong Creek, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19313,16 +19241,14 @@
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Centuria Capital Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Centuria Capital Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19398,16 +19324,14 @@
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Charter Hall's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Charter Hall's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19479,16 +19403,14 @@
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Community Housing Limited's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Community Housing Limited's role in delivering community and affordable housing across Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19564,16 +19486,14 @@
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Costa Property Group's pipeline, especially alongside Watermark in Armstrong Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Costa Property Group's active presence in Geelong and Armstrong Creek, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19649,16 +19569,14 @@
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Creation Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Creation Homes' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19730,16 +19648,14 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Crystal Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Crystal Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19811,16 +19727,14 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit C Street Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given C Street Projects' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19896,16 +19810,14 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Dahua Group Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Dahua Group Australia's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -19981,16 +19893,14 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit DealCorp's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given DealCorp's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20062,16 +19972,14 @@
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Dennis Family Corporation's pipeline, especially alongside Ashbury in Armstrong Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Dennis Family Corporation's active presence in Geelong and Armstrong Creek, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20147,16 +20055,14 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Development Edge's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Development Edge's active presence in Bendigo and Shepparton, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20228,16 +20134,14 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Development Victoria's pipeline, especially alongside Silverbrook in Mount Duneed:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Development Victoria's active presence in Geelong, Bendigo and Ballarat, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20313,16 +20217,14 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Dexus' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Dexus' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20398,16 +20300,14 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit DM Property's pipeline, especially alongside Uptown in Shepparton North:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given DM Property's active presence in Shepparton, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20483,16 +20383,14 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit ESR Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given ESR Australia's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20568,16 +20466,14 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Evolve Development's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Evolve Development's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20653,16 +20549,14 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit the Exford Waters team's pipeline, especially alongside Exford Waters in Weir Views:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given the Exford Waters team's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20738,16 +20632,14 @@
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Far East Consortium Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Far East Consortium Australia's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20819,16 +20711,14 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Frasers Property Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Frasers Property Australia's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20904,16 +20794,14 @@
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Gersh Investment Partners' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Gersh Investment Partners' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -20985,16 +20873,14 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Gill Family Corp's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Gill Family Corp's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21070,16 +20956,14 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Glenvill Homes' pipeline, especially alongside Ashbury in Armstrong Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Glenvill Homes' active presence in Geelong and Armstrong Creek, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21155,16 +21039,14 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Golden Age Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Golden Age Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21236,16 +21118,14 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Goldfields' pipeline, especially alongside Parkers Grove in Shepparton:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Goldfields' active presence in Shepparton, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21321,16 +21201,14 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Goodman Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Goodman Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21406,16 +21284,14 @@
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit GPT Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given GPT Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21491,16 +21367,14 @@
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Growland Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Growland Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21576,16 +21450,14 @@
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Gull &amp; Co's pipeline, especially alongside Avenue Hill in Ballarat:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Gull &amp; Co's active presence in Ballarat, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21657,16 +21529,14 @@
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit GURNER's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given GURNER's active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21742,16 +21612,14 @@
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hamilton Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Hamilton Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21827,16 +21695,14 @@
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hamton Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Hamton Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21912,16 +21778,14 @@
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hengyi Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Hengyi Australia's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -21997,16 +21861,14 @@
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hickory's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Hickory's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22082,16 +21944,14 @@
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Holder East's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Holder East's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22163,16 +22023,14 @@
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Homes Victoria's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Homes Victoria's role in delivering new homes across Melbourne's growth areas and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22248,16 +22106,14 @@
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Housing Choices Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Housing Choices Australia's role in delivering community and affordable housing across Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22333,16 +22189,14 @@
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit HousingFirst's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given HousingFirst's role in delivering community and affordable housing across Melbourne, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22414,16 +22268,14 @@
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hub Property Group's pipeline, especially alongside Balmoral Quay in Rippleside:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Hub Property Group's active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22495,16 +22347,14 @@
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hudson Ridge Builders' pipeline, especially alongside Aurora in Ballarat East:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Hudson Ridge Builders' active presence in Ballarat, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22580,16 +22430,14 @@
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Huntly Property Holdings' pipeline, especially alongside Provenance in Huntly:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Huntly Property Holdings' active presence in Bendigo, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22657,16 +22505,14 @@
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hygge Property's pipeline, especially alongside The Bottleworks in Geelong:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Hygge Property's active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22742,16 +22588,14 @@
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit ICD Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given ICD Property's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22827,16 +22671,14 @@
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit IDA's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given IDA's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22912,16 +22754,14 @@
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit ID_Land's pipeline, especially alongside Watermark in Armstrong Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given ID_Land's active presence in Geelong and Armstrong Creek, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -22993,16 +22833,14 @@
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Ingenia Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Ingenia Communities' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23078,16 +22916,14 @@
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Integra Group's pipeline, especially alongside Viewpoint Bendigo in Huntly:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Integra Group's active presence in Bendigo and Ballarat, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23163,16 +22999,14 @@
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Intrapac Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Intrapac Property's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23248,16 +23082,14 @@
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Jaydo Construction's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Jaydo Construction's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23321,16 +23153,14 @@
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Jayland Group's pipeline, especially alongside Central Park in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Jayland Group's active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23406,16 +23236,14 @@
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Jinding's pipeline, especially alongside Broadstead in Kilmore:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Jinding's active presence in Kilmore, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23491,16 +23319,14 @@
       </c>
       <c r="K88" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Kataland's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Kataland's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23572,16 +23398,14 @@
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Kode Living's pipeline, especially alongside Dream Ballarat in Sebastopol:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Kode Living's active presence in Ballarat, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23657,16 +23481,14 @@
       </c>
       <c r="K90" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Koham Property's pipeline, especially alongside Heritage Estate in Moe:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Koham Property's active presence in Moe, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23742,16 +23564,14 @@
       </c>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Kokoda Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Kokoda Property's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23827,16 +23647,14 @@
       </c>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit LandGipps' pipeline, especially alongside Mitchell Grove in Moe:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given LandGipps' active presence in Moe, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23908,16 +23726,14 @@
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Landmack Developments' pipeline, especially alongside Carringum Ballarat in Winter Valley:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Landmack Developments' active presence in Ballarat, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -23993,16 +23809,14 @@
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Landream's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Landream's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24070,16 +23884,14 @@
       </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lauders Group's pipeline, especially alongside Glenmore in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Lauders Group's active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24155,16 +23967,14 @@
       </c>
       <c r="K96" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Launch Housing's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Launch Housing's role in delivering housing for people experiencing homelessness across Melbourne, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24236,16 +24046,14 @@
       </c>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit LBDG Developer's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given LBDG Developer's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24317,16 +24125,14 @@
       </c>
       <c r="K98" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lendlease's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Lendlease's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24402,16 +24208,14 @@
       </c>
       <c r="K99" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lifestyle Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Lifestyle Communities' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24483,16 +24287,14 @@
       </c>
       <c r="K100" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Little Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Little Projects' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24564,16 +24366,14 @@
       </c>
       <c r="K101" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit LK Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given LK Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24645,16 +24445,14 @@
       </c>
       <c r="K102" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Local Residential's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Local Residential's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24730,16 +24528,14 @@
       </c>
       <c r="K103" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lotus Living's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Lotus Living's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24815,16 +24611,14 @@
       </c>
       <c r="K104" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lowe Living's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Lowe Living's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24896,16 +24690,14 @@
       </c>
       <c r="K105" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Maax Global's pipeline, especially alongside Creekview at Dalgona in Mount Duneed:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Maax Global's active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -24981,16 +24773,14 @@
       </c>
       <c r="K106" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit MAB Corporation's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given MAB Corporation's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25066,16 +24856,14 @@
       </c>
       <c r="K107" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Marlton Group's pipeline, especially alongside Montana in Kilmore:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Marlton Group's active presence in Kilmore, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25151,16 +24939,14 @@
       </c>
       <c r="K108" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit McMullin's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given McMullin's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25236,16 +25022,14 @@
       </c>
       <c r="K109" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Melbournia Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Melbournia Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25321,16 +25105,14 @@
       </c>
       <c r="K110" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit MetDev's pipeline, especially alongside Provenance in Huntly:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given MetDev's active presence in Bendigo, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25406,16 +25188,14 @@
       </c>
       <c r="K111" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Metricon Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Metricon Homes' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25491,16 +25271,14 @@
       </c>
       <c r="K112" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Milieu's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Milieu's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25576,16 +25354,14 @@
       </c>
       <c r="K113" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Mirvac's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Mirvac's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25657,16 +25433,14 @@
       </c>
       <c r="K114" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Miura Group's pipeline, especially alongside Beveridge Central:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Miura Group's active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25742,16 +25516,14 @@
       </c>
       <c r="K115" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Monash Views' pipeline, especially alongside Monash Views in Newborough:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Monash Views' active presence in Moe and Newborough, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25827,16 +25599,14 @@
       </c>
       <c r="K116" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Monno's pipeline, especially alongside Stella Maris in Rippleside:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Monno's active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25912,16 +25682,14 @@
       </c>
       <c r="K117" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Moremac Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Moremac Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -25997,16 +25765,14 @@
       </c>
       <c r="K118" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Morgan &amp; Griffin's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Morgan &amp; Griffin's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26082,16 +25848,14 @@
       </c>
       <c r="K119" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Neometro's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Neometro's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26163,16 +25927,14 @@
       </c>
       <c r="K120" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Newland Developers' pipeline, especially alongside Mandalay in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Newland Developers' active presence in Geelong, Beveridge and Armstrong Creek, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26248,16 +26010,14 @@
       </c>
       <c r="K121" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Nexus Developments' pipeline, especially alongside The Clan in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Nexus Developments' active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26329,16 +26089,14 @@
       </c>
       <c r="K122" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Nightingale Housing's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Nightingale Housing's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26410,16 +26168,14 @@
       </c>
       <c r="K123" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Oakbridge Developments' pipeline, especially alongside The Avenue in Flora Hill:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Oakbridge Developments' active presence in Bendigo, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26491,16 +26247,14 @@
       </c>
       <c r="K124" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Okeland Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Okeland Communities' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26576,16 +26330,14 @@
       </c>
       <c r="K125" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Oreana's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Oreana's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26661,16 +26413,14 @@
       </c>
       <c r="K126" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Orion International Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Orion International Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26746,16 +26496,14 @@
       </c>
       <c r="K127" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit OSK Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given OSK Property's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26831,16 +26579,14 @@
       </c>
       <c r="K128" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit OYOB Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given OYOB Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -26916,16 +26662,14 @@
       </c>
       <c r="K129" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pace Development Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Pace Development Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27001,16 +26745,14 @@
       </c>
       <c r="K130" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Parklea's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Parklea's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27086,16 +26828,14 @@
       </c>
       <c r="K131" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pask Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Pask Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27171,16 +26911,14 @@
       </c>
       <c r="K132" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit PDG Corporation's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given PDG Corporation's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27256,16 +26994,14 @@
       </c>
       <c r="K133" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Peet's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Peet's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27341,16 +27077,14 @@
       </c>
       <c r="K134" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pellicano's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Pellicano's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27426,16 +27160,14 @@
       </c>
       <c r="K135" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pelligra Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Pelligra Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27511,16 +27243,14 @@
       </c>
       <c r="K136" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Perri Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Perri Projects' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27596,16 +27326,14 @@
       </c>
       <c r="K137" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Piccolo's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Piccolo's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27681,16 +27409,14 @@
       </c>
       <c r="K138" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Prime Edition's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Prime Edition's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27754,16 +27480,14 @@
       </c>
       <c r="K139" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Providence Properties' pipeline, especially alongside The Stables Townhomes in Kilmore:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Providence Properties' active presence in Kilmore, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27839,16 +27563,14 @@
       </c>
       <c r="K140" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Quintessential's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Quintessential's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -27924,16 +27646,14 @@
       </c>
       <c r="K141" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Ramsey Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Ramsey Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28009,16 +27729,14 @@
       </c>
       <c r="K142" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Resimax Group's pipeline, especially alongside Talisen in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Resimax Group's active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28094,16 +27812,14 @@
       </c>
       <c r="K143" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Resi Ventures' pipeline, especially alongside Timbarra in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Resi Ventures' active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28179,16 +27895,14 @@
       </c>
       <c r="K144" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Risland's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Risland's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28264,16 +27978,14 @@
       </c>
       <c r="K145" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Riverlee's pipeline, especially alongside Lovely Banks:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Riverlee's active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28349,16 +28061,14 @@
       </c>
       <c r="K146" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit RW Developments' pipeline, especially alongside Parkview in Kilmore:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given RW Developments' active presence in Kilmore, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28434,16 +28144,14 @@
       </c>
       <c r="K147" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Salta Properties' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Salta Properties' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28519,16 +28227,14 @@
       </c>
       <c r="K148" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Salvo Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Salvo Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28604,16 +28310,14 @@
       </c>
       <c r="K149" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Satterley's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Satterley's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28681,16 +28385,14 @@
       </c>
       <c r="K150" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Scannell Properties' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Scannell Properties' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28762,16 +28464,14 @@
       </c>
       <c r="K151" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Seebeck Group Enterprise's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Seebeck Group Enterprise's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28847,16 +28547,14 @@
       </c>
       <c r="K152" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sentinel's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Sentinel's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -28928,16 +28626,14 @@
       </c>
       <c r="K153" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Serenitas Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Serenitas Management's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29013,16 +28709,14 @@
       </c>
       <c r="K154" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit SIG Group's pipeline, especially alongside Merri Park in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given SIG Group's active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29098,16 +28792,14 @@
       </c>
       <c r="K155" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit SightStone's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given SightStone's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29183,16 +28875,14 @@
       </c>
       <c r="K156" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Simonds Homes Victoria's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Simonds Homes Victoria's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29268,16 +28958,14 @@
       </c>
       <c r="K157" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sinclair Brook's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Sinclair Brook's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29353,16 +29041,14 @@
       </c>
       <c r="K158" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit SJD Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given SJD Homes' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29438,16 +29124,14 @@
       </c>
       <c r="K159" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit SOHO Living's pipeline, especially alongside The Greens at Mandalay in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given SOHO Living's active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29523,16 +29207,14 @@
       </c>
       <c r="K160" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Solovey's pipeline, especially alongside North Quarter in Newborough:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Solovey's active presence in Moe and Newborough, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29608,16 +29290,14 @@
       </c>
       <c r="K161" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Southern Sustainable Developments' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Southern Sustainable Developments' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29689,16 +29369,14 @@
       </c>
       <c r="K162" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Springtree's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Springtree's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29770,16 +29448,14 @@
       </c>
       <c r="K163" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit SP Setia Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given SP Setia Australia's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29855,16 +29531,14 @@
       </c>
       <c r="K164" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Star Investment Group's pipeline, especially alongside Lake Narracan Resort:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Star Investment Group's active presence in Moe, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -29940,16 +29614,14 @@
       </c>
       <c r="K165" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sterling Global's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Sterling Global's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30025,16 +29697,14 @@
       </c>
       <c r="K166" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Stockland's pipeline, especially alongside Lyra in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Stockland's active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30106,16 +29776,14 @@
       </c>
       <c r="K167" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Storehouse Capital's pipeline, especially alongside Mattana in Mount Duneed:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Storehouse Capital's active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30191,16 +29859,14 @@
       </c>
       <c r="K168" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sunkin Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Sunkin Property Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30276,16 +29942,14 @@
       </c>
       <c r="K169" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit SYP Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given SYP Property's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30361,16 +30025,14 @@
       </c>
       <c r="K170" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit The Corcoris Group's pipeline, especially alongside Ooranya in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given The Corcoris Group's active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30446,16 +30108,14 @@
       </c>
       <c r="K171" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit The Village Building Company's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given The Village Building Company's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30527,16 +30187,14 @@
       </c>
       <c r="K172" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Three Thirds Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Three Thirds Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30612,16 +30270,14 @@
       </c>
       <c r="K173" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Time &amp; Place's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Time &amp; Place's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30697,16 +30353,14 @@
       </c>
       <c r="K174" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Tripleton's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Tripleton's active presence in Geelong, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30782,16 +30436,14 @@
       </c>
       <c r="K175" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit UD Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given UD Australia's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30867,16 +30519,14 @@
       </c>
       <c r="K176" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Up Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Up Property's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -30948,16 +30598,14 @@
       </c>
       <c r="K177" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Urban Land Developments' pipeline, especially alongside Central Walk in Drysdale:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Urban Land Developments' active presence in Geelong and Drysdale, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -31033,16 +30681,14 @@
       </c>
       <c r="K178" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Urban Land Projects' pipeline, especially alongside The North Quarter in Shepparton:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Urban Land Projects' active presence in Shepparton, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -31118,16 +30764,14 @@
       </c>
       <c r="K179" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Urbex's pipeline, especially alongside Mandalay in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Urbex's active presence in Beveridge, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -31203,16 +30847,14 @@
       </c>
       <c r="K180" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Vicinity Centres' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Vicinity Centres' active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -31288,16 +30930,14 @@
       </c>
       <c r="K181" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Villawood Properties' pipeline, especially alongside Armstrong in Mount Duneed:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Villawood Properties' active presence in Geelong and Bendigo, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -31373,16 +31013,14 @@
       </c>
       <c r="K182" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Wel.Co's pipeline, especially alongside Harlowe Bendigo in Huntly:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Wel.Co's active presence in Bendigo, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -31458,16 +31096,14 @@
       </c>
       <c r="K183" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Wingate's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Wingate's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -31543,16 +31179,14 @@
       </c>
       <c r="K184" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit Wolfdene's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given Wolfdene's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -31624,16 +31258,14 @@
       </c>
       <c r="K185" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit XWISE Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given XWISE Group's active presence across Melbourne's growth corridors and regional Victoria, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC
@@ -31709,16 +31341,14 @@
       </c>
       <c r="K186" s="3" t="inlineStr">
         <is>
-          <t>Hi Acquisition Team,
-My name is Inder Sandhu with Crown Real Estate Agents. I specialise in development land across Melbourne's western and northern growth corridors and regional Victoria.
-I have development sites available across Wollert, Beveridge, Tarneit, Geelong, Deanside, Bonnie Brook, Fraser Rise and Truganina:
+          <t>Hi team,
+Quick one. I'm representing several development sites across Melbourne's north and west that may suit YourLand's pipeline, especially alongside The Last Piece in Golden Square:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
 * About 50 acres of investigation-area land.
-Given YourLand's active presence in Bendigo, I believe these sites would be a strong fit for your acquisitions pipeline.
-Could you please direct me to the appropriate contact in your acquisitions department so I can share further details?
-If you'd rather not hear from me about sites, just let me know and I won't contact you again.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
 Inder Sandhu
 Principal /OIEC

</xml_diff>

<commit_message>
Match the outreach message to the user's final layout
Drop the blank lines the user's version doesn't have, and spell
"authorised" the Australian way in the disclaimer.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -16340,7 +16340,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -16423,7 +16423,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -16502,7 +16502,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -16585,7 +16585,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -16664,7 +16664,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -16747,7 +16747,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -16830,7 +16830,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
@@ -16909,7 +16909,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -16984,7 +16984,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
@@ -17067,7 +17067,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -17150,7 +17150,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
@@ -17233,7 +17233,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -17316,7 +17316,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -17399,7 +17399,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -17478,7 +17478,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
@@ -17561,7 +17561,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
@@ -17640,7 +17640,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
@@ -17723,7 +17723,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -17806,7 +17806,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
@@ -17885,7 +17885,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -17964,7 +17964,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -18039,7 +18039,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -18118,7 +18118,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -18201,7 +18201,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -18284,7 +18284,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -18367,7 +18367,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
@@ -18450,7 +18450,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
@@ -18529,7 +18529,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
@@ -18608,7 +18608,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
@@ -18691,7 +18691,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
@@ -18770,7 +18770,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -18853,7 +18853,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
@@ -18932,7 +18932,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -19015,7 +19015,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -19098,7 +19098,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -19181,7 +19181,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -19260,7 +19260,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -19343,7 +19343,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -19422,7 +19422,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -19505,7 +19505,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr">
@@ -19588,7 +19588,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -19667,7 +19667,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -19746,7 +19746,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr">
@@ -19829,7 +19829,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -19912,7 +19912,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr">
@@ -19991,7 +19991,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
@@ -20074,7 +20074,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L48" s="2" t="inlineStr">
@@ -20153,7 +20153,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
@@ -20236,7 +20236,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -20319,7 +20319,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
@@ -20402,7 +20402,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -20485,7 +20485,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
@@ -20568,7 +20568,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
@@ -20651,7 +20651,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
@@ -20730,7 +20730,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
@@ -20813,7 +20813,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
@@ -20892,7 +20892,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L58" s="2" t="inlineStr">
@@ -20975,7 +20975,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L59" s="2" t="inlineStr">
@@ -21058,7 +21058,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
@@ -21137,7 +21137,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
@@ -21220,7 +21220,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
@@ -21303,7 +21303,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
@@ -21386,7 +21386,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
@@ -21469,7 +21469,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
@@ -21548,7 +21548,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
@@ -21631,7 +21631,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
@@ -21714,7 +21714,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
@@ -21797,7 +21797,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
@@ -21880,7 +21880,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
@@ -21963,7 +21963,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
@@ -22042,7 +22042,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
@@ -22125,7 +22125,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
@@ -22208,7 +22208,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
@@ -22287,7 +22287,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L75" s="2" t="inlineStr">
@@ -22366,7 +22366,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr">
@@ -22449,7 +22449,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr">
@@ -22524,7 +22524,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
@@ -22607,7 +22607,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L79" s="2" t="inlineStr">
@@ -22690,7 +22690,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
@@ -22773,7 +22773,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">
@@ -22852,7 +22852,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L82" s="2" t="inlineStr">
@@ -22935,7 +22935,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L83" s="2" t="inlineStr">
@@ -23018,7 +23018,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L84" s="2" t="inlineStr">
@@ -23101,7 +23101,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L85" s="2" t="inlineStr">
@@ -23172,7 +23172,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr">
@@ -23255,7 +23255,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L87" s="2" t="inlineStr">
@@ -23338,7 +23338,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L88" s="2" t="inlineStr">
@@ -23417,7 +23417,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L89" s="2" t="inlineStr">
@@ -23500,7 +23500,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L90" s="2" t="inlineStr">
@@ -23583,7 +23583,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L91" s="2" t="inlineStr">
@@ -23666,7 +23666,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr">
@@ -23745,7 +23745,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L93" s="2" t="inlineStr">
@@ -23828,7 +23828,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr">
@@ -23903,7 +23903,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr">
@@ -23986,7 +23986,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L96" s="2" t="inlineStr">
@@ -24065,7 +24065,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L97" s="2" t="inlineStr">
@@ -24144,7 +24144,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L98" s="2" t="inlineStr">
@@ -24227,7 +24227,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L99" s="2" t="inlineStr">
@@ -24306,7 +24306,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L100" s="2" t="inlineStr">
@@ -24385,7 +24385,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L101" s="2" t="inlineStr">
@@ -24464,7 +24464,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L102" s="2" t="inlineStr">
@@ -24547,7 +24547,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L103" s="2" t="inlineStr">
@@ -24630,7 +24630,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L104" s="2" t="inlineStr">
@@ -24709,7 +24709,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L105" s="2" t="inlineStr">
@@ -24792,7 +24792,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L106" s="2" t="inlineStr">
@@ -24875,7 +24875,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L107" s="2" t="inlineStr">
@@ -24958,7 +24958,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L108" s="2" t="inlineStr">
@@ -25041,7 +25041,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L109" s="2" t="inlineStr">
@@ -25124,7 +25124,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L110" s="2" t="inlineStr">
@@ -25207,7 +25207,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L111" s="2" t="inlineStr">
@@ -25290,7 +25290,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L112" s="2" t="inlineStr">
@@ -25373,7 +25373,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L113" s="2" t="inlineStr">
@@ -25452,7 +25452,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L114" s="2" t="inlineStr">
@@ -25535,7 +25535,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L115" s="2" t="inlineStr">
@@ -25618,7 +25618,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L116" s="2" t="inlineStr">
@@ -25701,7 +25701,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L117" s="2" t="inlineStr">
@@ -25784,7 +25784,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L118" s="2" t="inlineStr">
@@ -25867,7 +25867,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L119" s="2" t="inlineStr">
@@ -25946,7 +25946,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L120" s="2" t="inlineStr">
@@ -26029,7 +26029,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L121" s="2" t="inlineStr">
@@ -26108,7 +26108,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L122" s="2" t="inlineStr">
@@ -26187,7 +26187,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L123" s="2" t="inlineStr">
@@ -26266,7 +26266,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L124" s="2" t="inlineStr">
@@ -26349,7 +26349,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L125" s="2" t="inlineStr">
@@ -26432,7 +26432,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L126" s="2" t="inlineStr">
@@ -26515,7 +26515,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L127" s="2" t="inlineStr">
@@ -26598,7 +26598,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L128" s="2" t="inlineStr">
@@ -26681,7 +26681,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L129" s="2" t="inlineStr">
@@ -26764,7 +26764,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L130" s="2" t="inlineStr">
@@ -26847,7 +26847,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L131" s="2" t="inlineStr">
@@ -26930,7 +26930,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L132" s="2" t="inlineStr">
@@ -27013,7 +27013,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L133" s="2" t="inlineStr">
@@ -27096,7 +27096,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L134" s="2" t="inlineStr">
@@ -27179,7 +27179,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L135" s="2" t="inlineStr">
@@ -27262,7 +27262,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L136" s="2" t="inlineStr">
@@ -27345,7 +27345,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L137" s="2" t="inlineStr">
@@ -27428,7 +27428,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L138" s="2" t="inlineStr">
@@ -27499,7 +27499,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L139" s="2" t="inlineStr">
@@ -27582,7 +27582,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L140" s="2" t="inlineStr">
@@ -27665,7 +27665,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L141" s="2" t="inlineStr">
@@ -27748,7 +27748,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L142" s="2" t="inlineStr">
@@ -27831,7 +27831,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr">
@@ -27914,7 +27914,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr">
@@ -27997,7 +27997,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L145" s="2" t="inlineStr">
@@ -28080,7 +28080,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L146" s="2" t="inlineStr">
@@ -28163,7 +28163,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L147" s="2" t="inlineStr">
@@ -28246,7 +28246,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L148" s="2" t="inlineStr">
@@ -28329,7 +28329,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L149" s="2" t="inlineStr">
@@ -28404,7 +28404,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L150" s="2" t="inlineStr">
@@ -28483,7 +28483,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L151" s="2" t="inlineStr">
@@ -28566,7 +28566,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L152" s="2" t="inlineStr">
@@ -28645,7 +28645,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L153" s="2" t="inlineStr">
@@ -28728,7 +28728,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L154" s="2" t="inlineStr">
@@ -28811,7 +28811,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L155" s="2" t="inlineStr">
@@ -28894,7 +28894,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L156" s="2" t="inlineStr">
@@ -28977,7 +28977,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L157" s="2" t="inlineStr">
@@ -29060,7 +29060,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L158" s="2" t="inlineStr">
@@ -29143,7 +29143,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L159" s="2" t="inlineStr">
@@ -29226,7 +29226,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L160" s="2" t="inlineStr">
@@ -29309,7 +29309,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L161" s="2" t="inlineStr">
@@ -29388,7 +29388,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L162" s="2" t="inlineStr">
@@ -29467,7 +29467,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L163" s="2" t="inlineStr">
@@ -29550,7 +29550,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L164" s="2" t="inlineStr">
@@ -29633,7 +29633,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L165" s="2" t="inlineStr">
@@ -29716,7 +29716,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L166" s="2" t="inlineStr">
@@ -29795,7 +29795,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L167" s="2" t="inlineStr">
@@ -29878,7 +29878,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L168" s="2" t="inlineStr">
@@ -29961,7 +29961,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L169" s="2" t="inlineStr">
@@ -30044,7 +30044,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L170" s="2" t="inlineStr">
@@ -30127,7 +30127,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L171" s="2" t="inlineStr">
@@ -30206,7 +30206,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L172" s="2" t="inlineStr">
@@ -30289,7 +30289,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L173" s="2" t="inlineStr">
@@ -30372,7 +30372,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L174" s="2" t="inlineStr">
@@ -30455,7 +30455,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L175" s="2" t="inlineStr">
@@ -30538,7 +30538,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L176" s="2" t="inlineStr">
@@ -30617,7 +30617,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L177" s="2" t="inlineStr">
@@ -30700,7 +30700,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L178" s="2" t="inlineStr">
@@ -30783,7 +30783,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L179" s="2" t="inlineStr">
@@ -30866,7 +30866,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L180" s="2" t="inlineStr">
@@ -30949,7 +30949,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L181" s="2" t="inlineStr">
@@ -31032,7 +31032,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L182" s="2" t="inlineStr">
@@ -31115,7 +31115,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L183" s="2" t="inlineStr">
@@ -31198,7 +31198,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L184" s="2" t="inlineStr">
@@ -31277,7 +31277,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L185" s="2" t="inlineStr">
@@ -31360,7 +31360,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L186" s="2" t="inlineStr">
@@ -31445,7 +31445,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L187" s="2" t="inlineStr">
@@ -31534,7 +31534,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L188" s="2" t="inlineStr">
@@ -31623,7 +31623,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L189" s="2" t="inlineStr">
@@ -31712,7 +31712,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L190" s="2" t="inlineStr">
@@ -31801,7 +31801,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L191" s="2" t="inlineStr">
@@ -31890,7 +31890,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L192" s="2" t="inlineStr">
@@ -31979,7 +31979,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -32068,7 +32068,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
@@ -32157,7 +32157,7 @@
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
 While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
-No binding agreements may be concluded via email without written confirmation by an authorized representative of Crown Real Estate Agents.</t>
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Final outreach wording: "Hi Acquisition team", tidier spacing, no web line
Matches the user's final draft: greeting, "50 acres under investigation
area", blank lines around the close, and no website line in the signature
(Gmail's connector turns it into a redirect link).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -16321,12 +16321,12 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit 3L Alliance's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -16335,7 +16335,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -16404,12 +16403,12 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Abiwood's pipeline, especially alongside Pinnacle Ballarat in Smythes Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -16418,7 +16417,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -16483,12 +16481,12 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit ABN Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -16497,7 +16495,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -16566,12 +16563,12 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Accord Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -16580,7 +16577,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -16645,12 +16641,12 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Mirrastone's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -16659,7 +16655,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -16728,12 +16723,12 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Aliro Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -16742,7 +16737,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -16811,12 +16805,12 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Allam Property Group's pipeline, especially alongside Alkyra in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -16825,7 +16819,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -16890,12 +16883,12 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Anthela GPH Developments' pipeline, especially alongside Evermore in Kilmore:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -16904,7 +16897,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -16965,12 +16957,12 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Antipodean Land Developments' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -16979,7 +16971,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17048,12 +17039,12 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit APD Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17062,7 +17053,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17131,12 +17121,12 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Arc Living's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17145,7 +17135,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17214,12 +17203,12 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Assemble Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17228,7 +17217,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17297,12 +17285,12 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit AVID Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17311,7 +17299,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17380,12 +17367,12 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Balcon Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17394,7 +17381,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17459,12 +17445,12 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bamfa Properties' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17473,7 +17459,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17542,12 +17527,12 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Banco Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17556,7 +17541,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17621,12 +17605,12 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Banner Asset Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17635,7 +17619,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17704,12 +17687,12 @@
       </c>
       <c r="K19" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Barks 33's pipeline, especially alongside Forest Ridge in Strathfieldsaye:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17718,7 +17701,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17787,12 +17769,12 @@
       </c>
       <c r="K20" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bauenort's pipeline, especially alongside Alto Ballarat in Winter Valley:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17801,7 +17783,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17866,12 +17847,12 @@
       </c>
       <c r="K21" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bayport's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17880,7 +17861,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -17945,12 +17925,12 @@
       </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Begley Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -17959,7 +17939,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18020,12 +17999,12 @@
       </c>
       <c r="K23" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bennett Williams' pipeline, especially alongside Heritage Estate in Moe:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18034,7 +18013,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18099,12 +18077,12 @@
       </c>
       <c r="K24" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Beulah's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18113,7 +18091,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18182,12 +18159,12 @@
       </c>
       <c r="K25" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bevan Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18196,7 +18173,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18265,12 +18241,12 @@
       </c>
       <c r="K26" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Birchgrove Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18279,7 +18255,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18348,12 +18323,12 @@
       </c>
       <c r="K27" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bisinella Developments' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18362,7 +18337,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18431,12 +18405,12 @@
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit BMD Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18445,7 +18419,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18510,12 +18483,12 @@
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bolton Clarke's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18524,7 +18497,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18589,12 +18561,12 @@
       </c>
       <c r="K30" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Brennan Development Group's pipeline, especially alongside Golden Grove Bendigo in Jackass Flat:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18603,7 +18575,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18672,12 +18643,12 @@
       </c>
       <c r="K31" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Brown Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18686,7 +18657,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18751,12 +18721,12 @@
       </c>
       <c r="K32" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Buildcap Development Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18765,7 +18735,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18834,12 +18803,12 @@
       </c>
       <c r="K33" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Burbank Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18848,7 +18817,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18913,12 +18881,12 @@
       </c>
       <c r="K34" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Cadence Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -18927,7 +18895,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -18996,12 +18963,12 @@
       </c>
       <c r="K35" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Carlisle Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19010,7 +18977,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19079,12 +19045,12 @@
       </c>
       <c r="K36" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Cedar Woods' pipeline, especially alongside Somerley in Corio:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19093,7 +19059,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19162,12 +19127,12 @@
       </c>
       <c r="K37" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Central Equity's pipeline, especially alongside Palomino in Armstrong Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19176,7 +19141,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19241,12 +19205,12 @@
       </c>
       <c r="K38" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Centuria Capital Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19255,7 +19219,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19324,12 +19287,12 @@
       </c>
       <c r="K39" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Charter Hall's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19338,7 +19301,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19403,12 +19365,12 @@
       </c>
       <c r="K40" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Community Housing Limited's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19417,7 +19379,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19486,12 +19447,12 @@
       </c>
       <c r="K41" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Costa Property Group's pipeline, especially alongside Watermark in Armstrong Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19500,7 +19461,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19569,12 +19529,12 @@
       </c>
       <c r="K42" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Creation Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19583,7 +19543,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19648,12 +19607,12 @@
       </c>
       <c r="K43" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Crystal Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19662,7 +19621,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19727,12 +19685,12 @@
       </c>
       <c r="K44" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit C Street Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19741,7 +19699,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19810,12 +19767,12 @@
       </c>
       <c r="K45" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Dahua Group Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19824,7 +19781,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19893,12 +19849,12 @@
       </c>
       <c r="K46" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit DealCorp's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19907,7 +19863,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -19972,12 +19927,12 @@
       </c>
       <c r="K47" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Dennis Family Corporation's pipeline, especially alongside Ashbury in Armstrong Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -19986,7 +19941,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20055,12 +20009,12 @@
       </c>
       <c r="K48" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Development Edge's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20069,7 +20023,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20134,12 +20087,12 @@
       </c>
       <c r="K49" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Development Victoria's pipeline, especially alongside Silverbrook in Mount Duneed:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20148,7 +20101,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20217,12 +20169,12 @@
       </c>
       <c r="K50" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Dexus' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20231,7 +20183,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20300,12 +20251,12 @@
       </c>
       <c r="K51" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit DM Property's pipeline, especially alongside Uptown in Shepparton North:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20314,7 +20265,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20383,12 +20333,12 @@
       </c>
       <c r="K52" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit ESR Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20397,7 +20347,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20466,12 +20415,12 @@
       </c>
       <c r="K53" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Evolve Development's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20480,7 +20429,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20549,12 +20497,12 @@
       </c>
       <c r="K54" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit the Exford Waters team's pipeline, especially alongside Exford Waters in Weir Views:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20563,7 +20511,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20632,12 +20579,12 @@
       </c>
       <c r="K55" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Far East Consortium Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20646,7 +20593,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20711,12 +20657,12 @@
       </c>
       <c r="K56" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Frasers Property Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20725,7 +20671,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20794,12 +20739,12 @@
       </c>
       <c r="K57" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Gersh Investment Partners' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20808,7 +20753,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20873,12 +20817,12 @@
       </c>
       <c r="K58" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Gill Family Corp's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20887,7 +20831,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -20956,12 +20899,12 @@
       </c>
       <c r="K59" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Glenvill Homes' pipeline, especially alongside Ashbury in Armstrong Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -20970,7 +20913,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21039,12 +20981,12 @@
       </c>
       <c r="K60" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Golden Age Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21053,7 +20995,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21118,12 +21059,12 @@
       </c>
       <c r="K61" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Goldfields' pipeline, especially alongside Parkers Grove in Shepparton:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21132,7 +21073,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21201,12 +21141,12 @@
       </c>
       <c r="K62" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Goodman Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21215,7 +21155,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21284,12 +21223,12 @@
       </c>
       <c r="K63" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit GPT Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21298,7 +21237,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21367,12 +21305,12 @@
       </c>
       <c r="K64" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Growland Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21381,7 +21319,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21450,12 +21387,12 @@
       </c>
       <c r="K65" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Gull &amp; Co's pipeline, especially alongside Avenue Hill in Ballarat:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21464,7 +21401,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21529,12 +21465,12 @@
       </c>
       <c r="K66" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit GURNER's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21543,7 +21479,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21612,12 +21547,12 @@
       </c>
       <c r="K67" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hamilton Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21626,7 +21561,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21695,12 +21629,12 @@
       </c>
       <c r="K68" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hamton Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21709,7 +21643,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21778,12 +21711,12 @@
       </c>
       <c r="K69" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hengyi Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21792,7 +21725,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21861,12 +21793,12 @@
       </c>
       <c r="K70" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hickory's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21875,7 +21807,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -21944,12 +21875,12 @@
       </c>
       <c r="K71" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Holder East's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -21958,7 +21889,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22023,12 +21953,12 @@
       </c>
       <c r="K72" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Homes Victoria's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22037,7 +21967,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22106,12 +22035,12 @@
       </c>
       <c r="K73" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Housing Choices Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22120,7 +22049,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22189,12 +22117,12 @@
       </c>
       <c r="K74" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit HousingFirst's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22203,7 +22131,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22268,12 +22195,12 @@
       </c>
       <c r="K75" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hub Property Group's pipeline, especially alongside Balmoral Quay in Rippleside:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22282,7 +22209,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22347,12 +22273,12 @@
       </c>
       <c r="K76" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hudson Ridge Builders' pipeline, especially alongside Aurora in Ballarat East:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22361,7 +22287,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22430,12 +22355,12 @@
       </c>
       <c r="K77" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Huntly Property Holdings' pipeline, especially alongside Provenance in Huntly:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22444,7 +22369,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22505,12 +22429,12 @@
       </c>
       <c r="K78" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hygge Property's pipeline, especially alongside The Bottleworks in Geelong:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22519,7 +22443,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22588,12 +22511,12 @@
       </c>
       <c r="K79" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit ICD Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22602,7 +22525,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22671,12 +22593,12 @@
       </c>
       <c r="K80" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit IDA's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22685,7 +22607,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22754,12 +22675,12 @@
       </c>
       <c r="K81" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit ID_Land's pipeline, especially alongside Watermark in Armstrong Creek:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22768,7 +22689,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22833,12 +22753,12 @@
       </c>
       <c r="K82" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Ingenia Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22847,7 +22767,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22916,12 +22835,12 @@
       </c>
       <c r="K83" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Integra Group's pipeline, especially alongside Viewpoint Bendigo in Huntly:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -22930,7 +22849,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -22999,12 +22917,12 @@
       </c>
       <c r="K84" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Intrapac Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23013,7 +22931,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23082,12 +22999,12 @@
       </c>
       <c r="K85" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Jaydo Construction's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23096,7 +23013,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23153,12 +23069,12 @@
       </c>
       <c r="K86" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Jayland Group's pipeline, especially alongside Central Park in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23167,7 +23083,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23236,12 +23151,12 @@
       </c>
       <c r="K87" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Jinding's pipeline, especially alongside Broadstead in Kilmore:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23250,7 +23165,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23319,12 +23233,12 @@
       </c>
       <c r="K88" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Kataland's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23333,7 +23247,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23398,12 +23311,12 @@
       </c>
       <c r="K89" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Kode Living's pipeline, especially alongside Dream Ballarat in Sebastopol:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23412,7 +23325,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23481,12 +23393,12 @@
       </c>
       <c r="K90" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Koham Property's pipeline, especially alongside Heritage Estate in Moe:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23495,7 +23407,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23564,12 +23475,12 @@
       </c>
       <c r="K91" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Kokoda Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23578,7 +23489,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23647,12 +23557,12 @@
       </c>
       <c r="K92" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit LandGipps' pipeline, especially alongside Mitchell Grove in Moe:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23661,7 +23571,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23726,12 +23635,12 @@
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Landmack Developments' pipeline, especially alongside Carringum Ballarat in Winter Valley:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23740,7 +23649,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23809,12 +23717,12 @@
       </c>
       <c r="K94" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Landream's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23823,7 +23731,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23884,12 +23791,12 @@
       </c>
       <c r="K95" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lauders Group's pipeline, especially alongside Glenmore in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23898,7 +23805,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -23967,12 +23873,12 @@
       </c>
       <c r="K96" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Launch Housing's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -23981,7 +23887,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24046,12 +23951,12 @@
       </c>
       <c r="K97" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit LBDG Developer's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24060,7 +23965,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24125,12 +24029,12 @@
       </c>
       <c r="K98" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lendlease's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24139,7 +24043,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24208,12 +24111,12 @@
       </c>
       <c r="K99" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lifestyle Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24222,7 +24125,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24287,12 +24189,12 @@
       </c>
       <c r="K100" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Little Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24301,7 +24203,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24366,12 +24267,12 @@
       </c>
       <c r="K101" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit LK Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24380,7 +24281,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24445,12 +24345,12 @@
       </c>
       <c r="K102" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Local Residential's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24459,7 +24359,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24528,12 +24427,12 @@
       </c>
       <c r="K103" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lotus Living's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24542,7 +24441,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24611,12 +24509,12 @@
       </c>
       <c r="K104" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lowe Living's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24625,7 +24523,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24690,12 +24587,12 @@
       </c>
       <c r="K105" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Maax Global's pipeline, especially alongside Creekview at Dalgona in Mount Duneed:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24704,7 +24601,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24773,12 +24669,12 @@
       </c>
       <c r="K106" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit MAB Corporation's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24787,7 +24683,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24856,12 +24751,12 @@
       </c>
       <c r="K107" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Marlton Group's pipeline, especially alongside Montana in Kilmore:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24870,7 +24765,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -24939,12 +24833,12 @@
       </c>
       <c r="K108" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit McMullin's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -24953,7 +24847,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25022,12 +24915,12 @@
       </c>
       <c r="K109" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Melbournia Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25036,7 +24929,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25105,12 +24997,12 @@
       </c>
       <c r="K110" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit MetDev's pipeline, especially alongside Provenance in Huntly:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25119,7 +25011,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25188,12 +25079,12 @@
       </c>
       <c r="K111" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Metricon Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25202,7 +25093,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25271,12 +25161,12 @@
       </c>
       <c r="K112" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Milieu's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25285,7 +25175,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25354,12 +25243,12 @@
       </c>
       <c r="K113" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Mirvac's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25368,7 +25257,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25433,12 +25321,12 @@
       </c>
       <c r="K114" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Miura Group's pipeline, especially alongside Beveridge Central:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25447,7 +25335,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25516,12 +25403,12 @@
       </c>
       <c r="K115" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Monash Views' pipeline, especially alongside Monash Views in Newborough:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25530,7 +25417,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25599,12 +25485,12 @@
       </c>
       <c r="K116" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Monno's pipeline, especially alongside Stella Maris in Rippleside:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25613,7 +25499,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25682,12 +25567,12 @@
       </c>
       <c r="K117" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Moremac Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25696,7 +25581,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25765,12 +25649,12 @@
       </c>
       <c r="K118" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Morgan &amp; Griffin's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25779,7 +25663,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25848,12 +25731,12 @@
       </c>
       <c r="K119" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Neometro's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25862,7 +25745,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -25927,12 +25809,12 @@
       </c>
       <c r="K120" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Newland Developers' pipeline, especially alongside Mandalay in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -25941,7 +25823,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26010,12 +25891,12 @@
       </c>
       <c r="K121" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Nexus Developments' pipeline, especially alongside The Clan in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26024,7 +25905,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26089,12 +25969,12 @@
       </c>
       <c r="K122" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Nightingale Housing's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26103,7 +25983,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26168,12 +26047,12 @@
       </c>
       <c r="K123" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Oakbridge Developments' pipeline, especially alongside The Avenue in Flora Hill:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26182,7 +26061,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26247,12 +26125,12 @@
       </c>
       <c r="K124" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Okeland Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26261,7 +26139,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26330,12 +26207,12 @@
       </c>
       <c r="K125" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Oreana's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26344,7 +26221,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26413,12 +26289,12 @@
       </c>
       <c r="K126" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Orion International Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26427,7 +26303,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26496,12 +26371,12 @@
       </c>
       <c r="K127" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit OSK Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26510,7 +26385,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26579,12 +26453,12 @@
       </c>
       <c r="K128" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit OYOB Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26593,7 +26467,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26662,12 +26535,12 @@
       </c>
       <c r="K129" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pace Development Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26676,7 +26549,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26745,12 +26617,12 @@
       </c>
       <c r="K130" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Parklea's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26759,7 +26631,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26828,12 +26699,12 @@
       </c>
       <c r="K131" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pask Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26842,7 +26713,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26911,12 +26781,12 @@
       </c>
       <c r="K132" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit PDG Corporation's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -26925,7 +26795,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -26994,12 +26863,12 @@
       </c>
       <c r="K133" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Peet's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27008,7 +26877,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27077,12 +26945,12 @@
       </c>
       <c r="K134" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pellicano's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27091,7 +26959,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27160,12 +27027,12 @@
       </c>
       <c r="K135" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pelligra Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27174,7 +27041,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27243,12 +27109,12 @@
       </c>
       <c r="K136" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Perri Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27257,7 +27123,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27326,12 +27191,12 @@
       </c>
       <c r="K137" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Piccolo's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27340,7 +27205,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27409,12 +27273,12 @@
       </c>
       <c r="K138" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Prime Edition's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27423,7 +27287,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27480,12 +27343,12 @@
       </c>
       <c r="K139" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Providence Properties' pipeline, especially alongside The Stables Townhomes in Kilmore:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27494,7 +27357,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27563,12 +27425,12 @@
       </c>
       <c r="K140" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Quintessential's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27577,7 +27439,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27646,12 +27507,12 @@
       </c>
       <c r="K141" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Ramsey Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27660,7 +27521,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27729,12 +27589,12 @@
       </c>
       <c r="K142" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Resimax Group's pipeline, especially alongside Talisen in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27743,7 +27603,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27812,12 +27671,12 @@
       </c>
       <c r="K143" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Resi Ventures' pipeline, especially alongside Timbarra in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27826,7 +27685,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27895,12 +27753,12 @@
       </c>
       <c r="K144" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Risland's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27909,7 +27767,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -27978,12 +27835,12 @@
       </c>
       <c r="K145" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Riverlee's pipeline, especially alongside Lovely Banks:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -27992,7 +27849,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28061,12 +27917,12 @@
       </c>
       <c r="K146" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit RW Developments' pipeline, especially alongside Parkview in Kilmore:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28075,7 +27931,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28144,12 +27999,12 @@
       </c>
       <c r="K147" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Salta Properties' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28158,7 +28013,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28227,12 +28081,12 @@
       </c>
       <c r="K148" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Salvo Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28241,7 +28095,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28310,12 +28163,12 @@
       </c>
       <c r="K149" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Satterley's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28324,7 +28177,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28385,12 +28237,12 @@
       </c>
       <c r="K150" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Scannell Properties' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28399,7 +28251,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28464,12 +28315,12 @@
       </c>
       <c r="K151" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Seebeck Group Enterprise's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28478,7 +28329,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28547,12 +28397,12 @@
       </c>
       <c r="K152" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sentinel's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28561,7 +28411,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28626,12 +28475,12 @@
       </c>
       <c r="K153" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Serenitas Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28640,7 +28489,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28709,12 +28557,12 @@
       </c>
       <c r="K154" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit SIG Group's pipeline, especially alongside Merri Park in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28723,7 +28571,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28792,12 +28639,12 @@
       </c>
       <c r="K155" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit SightStone's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28806,7 +28653,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28875,12 +28721,12 @@
       </c>
       <c r="K156" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Simonds Homes Victoria's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28889,7 +28735,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -28958,12 +28803,12 @@
       </c>
       <c r="K157" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sinclair Brook's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -28972,7 +28817,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29041,12 +28885,12 @@
       </c>
       <c r="K158" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit SJD Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29055,7 +28899,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29124,12 +28967,12 @@
       </c>
       <c r="K159" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit SOHO Living's pipeline, especially alongside The Greens at Mandalay in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29138,7 +28981,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29207,12 +29049,12 @@
       </c>
       <c r="K160" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Solovey's pipeline, especially alongside North Quarter in Newborough:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29221,7 +29063,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29290,12 +29131,12 @@
       </c>
       <c r="K161" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Southern Sustainable Developments' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29304,7 +29145,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29369,12 +29209,12 @@
       </c>
       <c r="K162" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Springtree's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29383,7 +29223,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29448,12 +29287,12 @@
       </c>
       <c r="K163" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit SP Setia Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29462,7 +29301,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29531,12 +29369,12 @@
       </c>
       <c r="K164" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Star Investment Group's pipeline, especially alongside Lake Narracan Resort:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29545,7 +29383,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29614,12 +29451,12 @@
       </c>
       <c r="K165" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sterling Global's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29628,7 +29465,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29697,12 +29533,12 @@
       </c>
       <c r="K166" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Stockland's pipeline, especially alongside Lyra in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29711,7 +29547,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29776,12 +29611,12 @@
       </c>
       <c r="K167" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Storehouse Capital's pipeline, especially alongside Mattana in Mount Duneed:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29790,7 +29625,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29859,12 +29693,12 @@
       </c>
       <c r="K168" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sunkin Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29873,7 +29707,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -29942,12 +29775,12 @@
       </c>
       <c r="K169" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit SYP Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -29956,7 +29789,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30025,12 +29857,12 @@
       </c>
       <c r="K170" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit The Corcoris Group's pipeline, especially alongside Ooranya in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30039,7 +29871,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30108,12 +29939,12 @@
       </c>
       <c r="K171" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit The Village Building Company's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30122,7 +29953,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30187,12 +30017,12 @@
       </c>
       <c r="K172" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Three Thirds Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30201,7 +30031,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30270,12 +30099,12 @@
       </c>
       <c r="K173" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Time &amp; Place's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30284,7 +30113,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30353,12 +30181,12 @@
       </c>
       <c r="K174" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Tripleton's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30367,7 +30195,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30436,12 +30263,12 @@
       </c>
       <c r="K175" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit UD Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30450,7 +30277,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30519,12 +30345,12 @@
       </c>
       <c r="K176" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Up Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30533,7 +30359,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30598,12 +30423,12 @@
       </c>
       <c r="K177" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Urban Land Developments' pipeline, especially alongside Central Walk in Drysdale:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30612,7 +30437,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30681,12 +30505,12 @@
       </c>
       <c r="K178" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Urban Land Projects' pipeline, especially alongside The North Quarter in Shepparton:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30695,7 +30519,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30764,12 +30587,12 @@
       </c>
       <c r="K179" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Urbex's pipeline, especially alongside Mandalay in Beveridge:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30778,7 +30601,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30847,12 +30669,12 @@
       </c>
       <c r="K180" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Vicinity Centres' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30861,7 +30683,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -30930,12 +30751,12 @@
       </c>
       <c r="K181" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Villawood Properties' pipeline, especially alongside Armstrong in Mount Duneed:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -30944,7 +30765,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31013,12 +30833,12 @@
       </c>
       <c r="K182" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Wel.Co's pipeline, especially alongside Harlowe Bendigo in Huntly:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -31027,7 +30847,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31096,12 +30915,12 @@
       </c>
       <c r="K183" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Wingate's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -31110,7 +30929,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31179,12 +30997,12 @@
       </c>
       <c r="K184" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit Wolfdene's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -31193,7 +31011,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31258,12 +31075,12 @@
       </c>
       <c r="K185" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit XWISE Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -31272,7 +31089,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31341,12 +31157,12 @@
       </c>
       <c r="K186" s="3" t="inlineStr">
         <is>
-          <t>Hi team,
+          <t>Hi Acquisition team,
 Quick one. I'm representing several development sites across Melbourne's north and west that may suit YourLand's pipeline, especially alongside The Last Piece in Golden Square:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
-* About 50 acres of investigation-area land.
+* 50 acres under investigation area.
 Who in acquisitions should I send the details to?
 If it's not a fit, just let me know and I won't follow up.
 Kind Regards,
@@ -31355,7 +31171,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31440,7 +31255,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31529,7 +31343,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31618,7 +31431,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31707,7 +31519,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31796,7 +31607,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31885,7 +31695,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -31974,7 +31783,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -32063,7 +31871,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
@@ -32152,7 +31959,6 @@
 CROWN REAL ESTATE AGENTS
 Phone no: 0484 926 324
 Inder@crownrea.com.au
-www.crownrea.com.au
 Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
 The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
 Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).

</xml_diff>

<commit_message>
Give developers without a named project their own opening line
Where the data has no project for "especially alongside", the message now
anchors on where the sites are instead (Wollert and Beveridge through to
Tarneit, Truganina and Geelong).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -16322,7 +16322,7 @@
       <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit 3L Alliance's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for 3L Alliance's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -16482,7 +16482,7 @@
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit ABN Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for ABN Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -16564,7 +16564,7 @@
       <c r="K5" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Accord Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Accord Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -16642,7 +16642,7 @@
       <c r="K6" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Mirrastone's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Mirrastone's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -16724,7 +16724,7 @@
       <c r="K7" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Aliro Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Aliro Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -16958,7 +16958,7 @@
       <c r="K10" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Antipodean Land Developments' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Antipodean Land Developments' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -17040,7 +17040,7 @@
       <c r="K11" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit APD Projects' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for APD Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -17122,7 +17122,7 @@
       <c r="K12" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Arc Living's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Arc Living's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -17204,7 +17204,7 @@
       <c r="K13" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Assemble Communities' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Assemble Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -17286,7 +17286,7 @@
       <c r="K14" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit AVID Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for AVID Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -17368,7 +17368,7 @@
       <c r="K15" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Balcon Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Balcon Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -17446,7 +17446,7 @@
       <c r="K16" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bamfa Properties' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Bamfa Properties' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -17528,7 +17528,7 @@
       <c r="K17" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Banco Management's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Banco Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -17606,7 +17606,7 @@
       <c r="K18" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Banner Asset Management's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Banner Asset Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -17848,7 +17848,7 @@
       <c r="K21" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bayport's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Bayport's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -17926,7 +17926,7 @@
       <c r="K22" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Begley Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Begley Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18078,7 +18078,7 @@
       <c r="K24" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Beulah's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Beulah's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18160,7 +18160,7 @@
       <c r="K25" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bevan Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Bevan Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18242,7 +18242,7 @@
       <c r="K26" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Birchgrove Property's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Birchgrove Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18324,7 +18324,7 @@
       <c r="K27" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bisinella Developments' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Bisinella Developments' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18406,7 +18406,7 @@
       <c r="K28" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit BMD Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for BMD Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18484,7 +18484,7 @@
       <c r="K29" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Bolton Clarke's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Bolton Clarke's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18644,7 +18644,7 @@
       <c r="K31" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Brown Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Brown Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18722,7 +18722,7 @@
       <c r="K32" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Buildcap Development Management's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Buildcap Development Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18804,7 +18804,7 @@
       <c r="K33" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Burbank Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Burbank Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18882,7 +18882,7 @@
       <c r="K34" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Cadence Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Cadence Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -18964,7 +18964,7 @@
       <c r="K35" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Carlisle Homes' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Carlisle Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -19206,7 +19206,7 @@
       <c r="K38" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Centuria Capital Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Centuria Capital Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -19288,7 +19288,7 @@
       <c r="K39" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Charter Hall's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Charter Hall's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -19366,7 +19366,7 @@
       <c r="K40" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Community Housing Limited's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Community Housing Limited's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -19530,7 +19530,7 @@
       <c r="K42" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Creation Homes' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Creation Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -19608,7 +19608,7 @@
       <c r="K43" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Crystal Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Crystal Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -19686,7 +19686,7 @@
       <c r="K44" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit C Street Projects' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for C Street Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -19768,7 +19768,7 @@
       <c r="K45" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Dahua Group Australia's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Dahua Group Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -19850,7 +19850,7 @@
       <c r="K46" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit DealCorp's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for DealCorp's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -20010,7 +20010,7 @@
       <c r="K48" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Development Edge's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Development Edge's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -20170,7 +20170,7 @@
       <c r="K50" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Dexus' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Dexus' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -20334,7 +20334,7 @@
       <c r="K52" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit ESR Australia's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for ESR Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -20416,7 +20416,7 @@
       <c r="K53" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Evolve Development's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Evolve Development's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -20580,7 +20580,7 @@
       <c r="K55" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Far East Consortium Australia's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Far East Consortium Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -20658,7 +20658,7 @@
       <c r="K56" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Frasers Property Australia's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Frasers Property Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -20740,7 +20740,7 @@
       <c r="K57" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Gersh Investment Partners' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Gersh Investment Partners' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -20818,7 +20818,7 @@
       <c r="K58" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Gill Family Corp's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Gill Family Corp's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -20982,7 +20982,7 @@
       <c r="K60" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Golden Age Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Golden Age Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -21142,7 +21142,7 @@
       <c r="K62" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Goodman Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Goodman Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -21224,7 +21224,7 @@
       <c r="K63" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit GPT Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for GPT Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -21306,7 +21306,7 @@
       <c r="K64" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Growland Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Growland Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -21466,7 +21466,7 @@
       <c r="K66" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit GURNER's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for GURNER's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -21548,7 +21548,7 @@
       <c r="K67" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hamilton Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Hamilton Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -21630,7 +21630,7 @@
       <c r="K68" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hamton Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Hamton Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -21712,7 +21712,7 @@
       <c r="K69" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hengyi Australia's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Hengyi Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -21794,7 +21794,7 @@
       <c r="K70" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Hickory's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Hickory's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -21876,7 +21876,7 @@
       <c r="K71" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Holder East's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Holder East's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -21954,7 +21954,7 @@
       <c r="K72" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Homes Victoria's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Homes Victoria's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -22036,7 +22036,7 @@
       <c r="K73" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Housing Choices Australia's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Housing Choices Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -22118,7 +22118,7 @@
       <c r="K74" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit HousingFirst's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for HousingFirst's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -22512,7 +22512,7 @@
       <c r="K79" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit ICD Property's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for ICD Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -22594,7 +22594,7 @@
       <c r="K80" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit IDA's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for IDA's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -22754,7 +22754,7 @@
       <c r="K82" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Ingenia Communities' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Ingenia Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -22918,7 +22918,7 @@
       <c r="K84" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Intrapac Property's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Intrapac Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -23000,7 +23000,7 @@
       <c r="K85" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Jaydo Construction's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Jaydo Construction's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -23234,7 +23234,7 @@
       <c r="K88" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Kataland's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Kataland's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -23476,7 +23476,7 @@
       <c r="K91" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Kokoda Property's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Kokoda Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -23718,7 +23718,7 @@
       <c r="K94" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Landream's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Landream's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -23874,7 +23874,7 @@
       <c r="K96" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Launch Housing's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Launch Housing's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -23952,7 +23952,7 @@
       <c r="K97" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit LBDG Developer's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for LBDG Developer's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -24030,7 +24030,7 @@
       <c r="K98" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lendlease's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Lendlease's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -24112,7 +24112,7 @@
       <c r="K99" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lifestyle Communities' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Lifestyle Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -24190,7 +24190,7 @@
       <c r="K100" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Little Projects' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Little Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -24268,7 +24268,7 @@
       <c r="K101" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit LK Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for LK Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -24346,7 +24346,7 @@
       <c r="K102" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Local Residential's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Local Residential's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -24428,7 +24428,7 @@
       <c r="K103" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lotus Living's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Lotus Living's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -24510,7 +24510,7 @@
       <c r="K104" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Lowe Living's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Lowe Living's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -24670,7 +24670,7 @@
       <c r="K106" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit MAB Corporation's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for MAB Corporation's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -24834,7 +24834,7 @@
       <c r="K108" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit McMullin's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for McMullin's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -24916,7 +24916,7 @@
       <c r="K109" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Melbournia Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Melbournia Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -25080,7 +25080,7 @@
       <c r="K111" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Metricon Homes' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Metricon Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -25162,7 +25162,7 @@
       <c r="K112" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Milieu's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Milieu's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -25244,7 +25244,7 @@
       <c r="K113" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Mirvac's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Mirvac's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -25568,7 +25568,7 @@
       <c r="K117" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Moremac Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Moremac Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -25650,7 +25650,7 @@
       <c r="K118" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Morgan &amp; Griffin's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Morgan &amp; Griffin's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -25732,7 +25732,7 @@
       <c r="K119" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Neometro's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Neometro's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -25970,7 +25970,7 @@
       <c r="K122" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Nightingale Housing's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Nightingale Housing's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26126,7 +26126,7 @@
       <c r="K124" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Okeland Communities' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Okeland Communities' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26208,7 +26208,7 @@
       <c r="K125" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Oreana's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Oreana's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26290,7 +26290,7 @@
       <c r="K126" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Orion International Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Orion International Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26372,7 +26372,7 @@
       <c r="K127" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit OSK Property's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for OSK Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26454,7 +26454,7 @@
       <c r="K128" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit OYOB Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for OYOB Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26536,7 +26536,7 @@
       <c r="K129" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pace Development Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Pace Development Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26618,7 +26618,7 @@
       <c r="K130" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Parklea's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Parklea's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26700,7 +26700,7 @@
       <c r="K131" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pask Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Pask Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26782,7 +26782,7 @@
       <c r="K132" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit PDG Corporation's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for PDG Corporation's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26864,7 +26864,7 @@
       <c r="K133" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Peet's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Peet's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -26946,7 +26946,7 @@
       <c r="K134" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pellicano's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Pellicano's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -27028,7 +27028,7 @@
       <c r="K135" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Pelligra Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Pelligra Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -27110,7 +27110,7 @@
       <c r="K136" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Perri Projects' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Perri Projects' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -27192,7 +27192,7 @@
       <c r="K137" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Piccolo's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Piccolo's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -27274,7 +27274,7 @@
       <c r="K138" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Prime Edition's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Prime Edition's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -27426,7 +27426,7 @@
       <c r="K140" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Quintessential's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Quintessential's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -27508,7 +27508,7 @@
       <c r="K141" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Ramsey Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Ramsey Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -27754,7 +27754,7 @@
       <c r="K144" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Risland's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Risland's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28000,7 +28000,7 @@
       <c r="K147" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Salta Properties' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Salta Properties' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28082,7 +28082,7 @@
       <c r="K148" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Salvo Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Salvo Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28164,7 +28164,7 @@
       <c r="K149" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Satterley's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Satterley's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28238,7 +28238,7 @@
       <c r="K150" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Scannell Properties' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Scannell Properties' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28316,7 +28316,7 @@
       <c r="K151" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Seebeck Group Enterprise's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Seebeck Group Enterprise's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28398,7 +28398,7 @@
       <c r="K152" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sentinel's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Sentinel's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28476,7 +28476,7 @@
       <c r="K153" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Serenitas Management's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Serenitas Management's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28640,7 +28640,7 @@
       <c r="K155" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit SightStone's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for SightStone's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28722,7 +28722,7 @@
       <c r="K156" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Simonds Homes Victoria's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Simonds Homes Victoria's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28804,7 +28804,7 @@
       <c r="K157" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sinclair Brook's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Sinclair Brook's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -28886,7 +28886,7 @@
       <c r="K158" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit SJD Homes' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for SJD Homes' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -29132,7 +29132,7 @@
       <c r="K161" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Southern Sustainable Developments' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Southern Sustainable Developments' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -29210,7 +29210,7 @@
       <c r="K162" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Springtree's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Springtree's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -29288,7 +29288,7 @@
       <c r="K163" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit SP Setia Australia's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for SP Setia Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -29452,7 +29452,7 @@
       <c r="K165" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sterling Global's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Sterling Global's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -29694,7 +29694,7 @@
       <c r="K168" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Sunkin Property Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Sunkin Property Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -29776,7 +29776,7 @@
       <c r="K169" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit SYP Property's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for SYP Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -29940,7 +29940,7 @@
       <c r="K171" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit The Village Building Company's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for The Village Building Company's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -30018,7 +30018,7 @@
       <c r="K172" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Three Thirds Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Three Thirds Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -30100,7 +30100,7 @@
       <c r="K173" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Time &amp; Place's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Time &amp; Place's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -30182,7 +30182,7 @@
       <c r="K174" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Tripleton's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Tripleton's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -30264,7 +30264,7 @@
       <c r="K175" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit UD Australia's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for UD Australia's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -30346,7 +30346,7 @@
       <c r="K176" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Up Property's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Up Property's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -30670,7 +30670,7 @@
       <c r="K180" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Vicinity Centres' pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Vicinity Centres' pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -30916,7 +30916,7 @@
       <c r="K183" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Wingate's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Wingate's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -30998,7 +30998,7 @@
       <c r="K184" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit Wolfdene's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for Wolfdene's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.
@@ -31076,7 +31076,7 @@
       <c r="K185" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing several development sites across Melbourne's north and west that may suit XWISE Group's pipeline:
+Quick one. I'm representing several development sites across Melbourne's north and west, from Wollert and Beveridge through to Tarneit, Truganina and Geelong, that could be a strong fit for XWISE Group's pipeline:
 * Shovel-ready residential and industrial.
 * Permit-approved townhouse sites, including one for 44 townhouses.
 * Childcare and townhouse sites, both raw and approved.

</xml_diff>

<commit_message>
Record who has been emailed on the Outreach tab
outreach_status.json logs the 3 October send (111 emails), the 10 the user
sent by hand, and the 43 addresses emailed before this campaign. The build
writes it into the Status column so nobody is contacted twice; rows still
"Not sent" are the contact-form-only organisations and the four selling
agents.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -16344,7 +16344,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr"/>
@@ -16426,7 +16426,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -16586,7 +16586,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr"/>
@@ -16746,7 +16746,7 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr"/>
@@ -16828,7 +16828,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr"/>
@@ -16906,7 +16906,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr"/>
@@ -16980,7 +16980,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr"/>
@@ -17062,7 +17062,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr"/>
@@ -17144,7 +17144,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr"/>
@@ -17226,7 +17226,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr"/>
@@ -17308,7 +17308,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr"/>
@@ -17390,7 +17390,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr"/>
@@ -17550,7 +17550,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr"/>
@@ -17792,7 +17792,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-02 (by Inder)</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr"/>
@@ -18100,7 +18100,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr"/>
@@ -18182,7 +18182,7 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr"/>
@@ -18264,7 +18264,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr"/>
@@ -18346,7 +18346,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr"/>
@@ -18428,7 +18428,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr"/>
@@ -18584,7 +18584,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr"/>
@@ -18666,7 +18666,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr"/>
@@ -18744,7 +18744,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr"/>
@@ -18826,7 +18826,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr"/>
@@ -18904,7 +18904,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr"/>
@@ -18986,7 +18986,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr"/>
@@ -19068,7 +19068,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr"/>
@@ -19150,7 +19150,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr"/>
@@ -19310,7 +19310,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr"/>
@@ -19470,7 +19470,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr"/>
@@ -19552,7 +19552,7 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr"/>
@@ -19708,7 +19708,7 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M44" s="2" t="inlineStr"/>
@@ -19790,7 +19790,7 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr"/>
@@ -19872,7 +19872,7 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr"/>
@@ -20032,7 +20032,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr"/>
@@ -20192,7 +20192,7 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr"/>
@@ -20274,7 +20274,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr"/>
@@ -20356,7 +20356,7 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03 (by Inder, earlier wording)</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr"/>
@@ -20438,7 +20438,7 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03 (by Inder, earlier wording)</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr"/>
@@ -20520,7 +20520,7 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03 (by Inder, earlier wording)</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr"/>
@@ -20602,7 +20602,7 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr"/>
@@ -20762,7 +20762,7 @@
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M57" s="2" t="inlineStr"/>
@@ -20840,7 +20840,7 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M58" s="2" t="inlineStr"/>
@@ -20922,7 +20922,7 @@
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M59" s="2" t="inlineStr"/>
@@ -21004,7 +21004,7 @@
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M60" s="2" t="inlineStr"/>
@@ -21082,7 +21082,7 @@
       </c>
       <c r="L61" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M61" s="2" t="inlineStr"/>
@@ -21164,7 +21164,7 @@
       </c>
       <c r="L62" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M62" s="2" t="inlineStr"/>
@@ -21246,7 +21246,7 @@
       </c>
       <c r="L63" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M63" s="2" t="inlineStr"/>
@@ -21328,7 +21328,7 @@
       </c>
       <c r="L64" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M64" s="2" t="inlineStr"/>
@@ -21410,7 +21410,7 @@
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M65" s="2" t="inlineStr"/>
@@ -21570,7 +21570,7 @@
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M67" s="2" t="inlineStr"/>
@@ -21652,7 +21652,7 @@
       </c>
       <c r="L68" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M68" s="2" t="inlineStr"/>
@@ -21734,7 +21734,7 @@
       </c>
       <c r="L69" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-02 (by Inder)</t>
         </is>
       </c>
       <c r="M69" s="2" t="inlineStr"/>
@@ -21816,7 +21816,7 @@
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M70" s="2" t="inlineStr"/>
@@ -21898,7 +21898,7 @@
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M71" s="2" t="inlineStr"/>
@@ -22058,7 +22058,7 @@
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M73" s="2" t="inlineStr"/>
@@ -22140,7 +22140,7 @@
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M74" s="2" t="inlineStr"/>
@@ -22218,7 +22218,7 @@
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M75" s="2" t="inlineStr"/>
@@ -22296,7 +22296,7 @@
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M76" s="2" t="inlineStr"/>
@@ -22378,7 +22378,7 @@
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M77" s="2" t="inlineStr"/>
@@ -22452,7 +22452,7 @@
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M78" s="2" t="inlineStr"/>
@@ -22534,7 +22534,7 @@
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M79" s="2" t="inlineStr"/>
@@ -22616,7 +22616,7 @@
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M80" s="2" t="inlineStr"/>
@@ -22698,7 +22698,7 @@
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M81" s="2" t="inlineStr"/>
@@ -22858,7 +22858,7 @@
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M83" s="2" t="inlineStr"/>
@@ -22940,7 +22940,7 @@
       </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M84" s="2" t="inlineStr"/>
@@ -23022,7 +23022,7 @@
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M85" s="2" t="inlineStr"/>
@@ -23174,7 +23174,7 @@
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M87" s="2" t="inlineStr"/>
@@ -23256,7 +23256,7 @@
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-02 (by Inder)</t>
         </is>
       </c>
       <c r="M88" s="2" t="inlineStr"/>
@@ -23334,7 +23334,7 @@
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M89" s="2" t="inlineStr"/>
@@ -23416,7 +23416,7 @@
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M90" s="2" t="inlineStr"/>
@@ -23498,7 +23498,7 @@
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M91" s="2" t="inlineStr"/>
@@ -23580,7 +23580,7 @@
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M92" s="2" t="inlineStr"/>
@@ -23740,7 +23740,7 @@
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M94" s="2" t="inlineStr"/>
@@ -23896,7 +23896,7 @@
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-02 (by Inder)</t>
         </is>
       </c>
       <c r="M96" s="2" t="inlineStr"/>
@@ -24134,7 +24134,7 @@
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M99" s="2" t="inlineStr"/>
@@ -24212,7 +24212,7 @@
       </c>
       <c r="L100" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M100" s="2" t="inlineStr"/>
@@ -24290,7 +24290,7 @@
       </c>
       <c r="L101" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M101" s="2" t="inlineStr"/>
@@ -24368,7 +24368,7 @@
       </c>
       <c r="L102" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M102" s="2" t="inlineStr"/>
@@ -24450,7 +24450,7 @@
       </c>
       <c r="L103" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M103" s="2" t="inlineStr"/>
@@ -24532,7 +24532,7 @@
       </c>
       <c r="L104" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M104" s="2" t="inlineStr"/>
@@ -24610,7 +24610,7 @@
       </c>
       <c r="L105" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M105" s="2" t="inlineStr"/>
@@ -24692,7 +24692,7 @@
       </c>
       <c r="L106" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M106" s="2" t="inlineStr"/>
@@ -24774,7 +24774,7 @@
       </c>
       <c r="L107" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M107" s="2" t="inlineStr"/>
@@ -24856,7 +24856,7 @@
       </c>
       <c r="L108" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M108" s="2" t="inlineStr"/>
@@ -24938,7 +24938,7 @@
       </c>
       <c r="L109" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M109" s="2" t="inlineStr"/>
@@ -25020,7 +25020,7 @@
       </c>
       <c r="L110" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M110" s="2" t="inlineStr"/>
@@ -25102,7 +25102,7 @@
       </c>
       <c r="L111" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M111" s="2" t="inlineStr"/>
@@ -25184,7 +25184,7 @@
       </c>
       <c r="L112" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M112" s="2" t="inlineStr"/>
@@ -25266,7 +25266,7 @@
       </c>
       <c r="L113" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03 (by Inder, earlier wording)</t>
         </is>
       </c>
       <c r="M113" s="2" t="inlineStr"/>
@@ -25344,7 +25344,7 @@
       </c>
       <c r="L114" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M114" s="2" t="inlineStr"/>
@@ -25426,7 +25426,7 @@
       </c>
       <c r="L115" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M115" s="2" t="inlineStr"/>
@@ -25508,7 +25508,7 @@
       </c>
       <c r="L116" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M116" s="2" t="inlineStr"/>
@@ -25590,7 +25590,7 @@
       </c>
       <c r="L117" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M117" s="2" t="inlineStr"/>
@@ -25672,7 +25672,7 @@
       </c>
       <c r="L118" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M118" s="2" t="inlineStr"/>
@@ -25754,7 +25754,7 @@
       </c>
       <c r="L119" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M119" s="2" t="inlineStr"/>
@@ -25832,7 +25832,7 @@
       </c>
       <c r="L120" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M120" s="2" t="inlineStr"/>
@@ -25914,7 +25914,7 @@
       </c>
       <c r="L121" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M121" s="2" t="inlineStr"/>
@@ -25992,7 +25992,7 @@
       </c>
       <c r="L122" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M122" s="2" t="inlineStr"/>
@@ -26070,7 +26070,7 @@
       </c>
       <c r="L123" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M123" s="2" t="inlineStr"/>
@@ -26230,7 +26230,7 @@
       </c>
       <c r="L125" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M125" s="2" t="inlineStr"/>
@@ -26312,7 +26312,7 @@
       </c>
       <c r="L126" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M126" s="2" t="inlineStr"/>
@@ -26394,7 +26394,7 @@
       </c>
       <c r="L127" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M127" s="2" t="inlineStr"/>
@@ -26476,7 +26476,7 @@
       </c>
       <c r="L128" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M128" s="2" t="inlineStr"/>
@@ -26558,7 +26558,7 @@
       </c>
       <c r="L129" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M129" s="2" t="inlineStr"/>
@@ -26640,7 +26640,7 @@
       </c>
       <c r="L130" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M130" s="2" t="inlineStr"/>
@@ -26722,7 +26722,7 @@
       </c>
       <c r="L131" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M131" s="2" t="inlineStr"/>
@@ -26804,7 +26804,7 @@
       </c>
       <c r="L132" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M132" s="2" t="inlineStr"/>
@@ -26886,7 +26886,7 @@
       </c>
       <c r="L133" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M133" s="2" t="inlineStr"/>
@@ -26968,7 +26968,7 @@
       </c>
       <c r="L134" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M134" s="2" t="inlineStr"/>
@@ -27050,7 +27050,7 @@
       </c>
       <c r="L135" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M135" s="2" t="inlineStr"/>
@@ -27132,7 +27132,7 @@
       </c>
       <c r="L136" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M136" s="2" t="inlineStr"/>
@@ -27214,7 +27214,7 @@
       </c>
       <c r="L137" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M137" s="2" t="inlineStr"/>
@@ -27296,7 +27296,7 @@
       </c>
       <c r="L138" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M138" s="2" t="inlineStr"/>
@@ -27448,7 +27448,7 @@
       </c>
       <c r="L140" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M140" s="2" t="inlineStr"/>
@@ -27530,7 +27530,7 @@
       </c>
       <c r="L141" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M141" s="2" t="inlineStr"/>
@@ -27612,7 +27612,7 @@
       </c>
       <c r="L142" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M142" s="2" t="inlineStr"/>
@@ -27694,7 +27694,7 @@
       </c>
       <c r="L143" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M143" s="2" t="inlineStr"/>
@@ -27776,7 +27776,7 @@
       </c>
       <c r="L144" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M144" s="2" t="inlineStr"/>
@@ -27858,7 +27858,7 @@
       </c>
       <c r="L145" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M145" s="2" t="inlineStr"/>
@@ -28022,7 +28022,7 @@
       </c>
       <c r="L147" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M147" s="2" t="inlineStr"/>
@@ -28104,7 +28104,7 @@
       </c>
       <c r="L148" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M148" s="2" t="inlineStr"/>
@@ -28186,7 +28186,7 @@
       </c>
       <c r="L149" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M149" s="2" t="inlineStr"/>
@@ -28338,7 +28338,7 @@
       </c>
       <c r="L151" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M151" s="2" t="inlineStr"/>
@@ -28420,7 +28420,7 @@
       </c>
       <c r="L152" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M152" s="2" t="inlineStr"/>
@@ -28498,7 +28498,7 @@
       </c>
       <c r="L153" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-02 (by Inder)</t>
         </is>
       </c>
       <c r="M153" s="2" t="inlineStr"/>
@@ -28580,7 +28580,7 @@
       </c>
       <c r="L154" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M154" s="2" t="inlineStr"/>
@@ -28662,7 +28662,7 @@
       </c>
       <c r="L155" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M155" s="2" t="inlineStr"/>
@@ -28744,7 +28744,7 @@
       </c>
       <c r="L156" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M156" s="2" t="inlineStr"/>
@@ -28826,7 +28826,7 @@
       </c>
       <c r="L157" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M157" s="2" t="inlineStr"/>
@@ -28908,7 +28908,7 @@
       </c>
       <c r="L158" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M158" s="2" t="inlineStr"/>
@@ -28990,7 +28990,7 @@
       </c>
       <c r="L159" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M159" s="2" t="inlineStr"/>
@@ -29072,7 +29072,7 @@
       </c>
       <c r="L160" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M160" s="2" t="inlineStr"/>
@@ -29154,7 +29154,7 @@
       </c>
       <c r="L161" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M161" s="2" t="inlineStr"/>
@@ -29310,7 +29310,7 @@
       </c>
       <c r="L163" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M163" s="2" t="inlineStr"/>
@@ -29392,7 +29392,7 @@
       </c>
       <c r="L164" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M164" s="2" t="inlineStr"/>
@@ -29474,7 +29474,7 @@
       </c>
       <c r="L165" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M165" s="2" t="inlineStr"/>
@@ -29556,7 +29556,7 @@
       </c>
       <c r="L166" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M166" s="2" t="inlineStr"/>
@@ -29716,7 +29716,7 @@
       </c>
       <c r="L168" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M168" s="2" t="inlineStr"/>
@@ -29798,7 +29798,7 @@
       </c>
       <c r="L169" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M169" s="2" t="inlineStr"/>
@@ -29880,7 +29880,7 @@
       </c>
       <c r="L170" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M170" s="2" t="inlineStr"/>
@@ -29962,7 +29962,7 @@
       </c>
       <c r="L171" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M171" s="2" t="inlineStr"/>
@@ -30040,7 +30040,7 @@
       </c>
       <c r="L172" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M172" s="2" t="inlineStr"/>
@@ -30122,7 +30122,7 @@
       </c>
       <c r="L173" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M173" s="2" t="inlineStr"/>
@@ -30204,7 +30204,7 @@
       </c>
       <c r="L174" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M174" s="2" t="inlineStr"/>
@@ -30286,7 +30286,7 @@
       </c>
       <c r="L175" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-02 (by Inder)</t>
         </is>
       </c>
       <c r="M175" s="2" t="inlineStr"/>
@@ -30368,7 +30368,7 @@
       </c>
       <c r="L176" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M176" s="2" t="inlineStr"/>
@@ -30528,7 +30528,7 @@
       </c>
       <c r="L178" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M178" s="2" t="inlineStr"/>
@@ -30610,7 +30610,7 @@
       </c>
       <c r="L179" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M179" s="2" t="inlineStr"/>
@@ -30692,7 +30692,7 @@
       </c>
       <c r="L180" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M180" s="2" t="inlineStr"/>
@@ -30774,7 +30774,7 @@
       </c>
       <c r="L181" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M181" s="2" t="inlineStr"/>
@@ -30856,7 +30856,7 @@
       </c>
       <c r="L182" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M182" s="2" t="inlineStr"/>
@@ -30938,7 +30938,7 @@
       </c>
       <c r="L183" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M183" s="2" t="inlineStr"/>
@@ -31020,7 +31020,7 @@
       </c>
       <c r="L184" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M184" s="2" t="inlineStr"/>
@@ -31098,7 +31098,7 @@
       </c>
       <c r="L185" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M185" s="2" t="inlineStr"/>
@@ -31180,7 +31180,7 @@
       </c>
       <c r="L186" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Emailed before this campaign</t>
         </is>
       </c>
       <c r="M186" s="2" t="inlineStr"/>
@@ -31264,7 +31264,7 @@
       </c>
       <c r="L187" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M187" s="2" t="inlineStr"/>
@@ -31352,7 +31352,7 @@
       </c>
       <c r="L188" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M188" s="2" t="inlineStr"/>
@@ -31440,7 +31440,7 @@
       </c>
       <c r="L189" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M189" s="2" t="inlineStr"/>
@@ -31528,7 +31528,7 @@
       </c>
       <c r="L190" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M190" s="2" t="inlineStr"/>
@@ -31616,7 +31616,7 @@
       </c>
       <c r="L191" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M191" s="2" t="inlineStr"/>
@@ -31704,7 +31704,7 @@
       </c>
       <c r="L192" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M192" s="2" t="inlineStr"/>
@@ -31792,7 +31792,7 @@
       </c>
       <c r="L193" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M193" s="2" t="inlineStr"/>
@@ -31880,7 +31880,7 @@
       </c>
       <c r="L194" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M194" s="2" t="inlineStr"/>
@@ -31968,7 +31968,7 @@
       </c>
       <c r="L195" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Sent 2026-10-03</t>
         </is>
       </c>
       <c r="M195" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Mark the four selling-agent drafts on the Outreach tab
Barks 33, Landmack, RW Developments and Storehouse Capital publish only
their selling agent's email, so each agent got a draft addressed to them
by name, naming the estate they sell and asking them to pass it on.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -17710,7 +17710,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03 (selling agent – asks them to pass it on)</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr"/>
@@ -23658,7 +23658,7 @@
       </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03 (selling agent – asks them to pass it on)</t>
         </is>
       </c>
       <c r="M93" s="2" t="inlineStr"/>
@@ -27940,7 +27940,7 @@
       </c>
       <c r="L146" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03 (selling agent – asks them to pass it on)</t>
         </is>
       </c>
       <c r="M146" s="2" t="inlineStr"/>
@@ -29634,7 +29634,7 @@
       </c>
       <c r="L167" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03 (selling agent – asks them to pass it on)</t>
         </is>
       </c>
       <c r="M167" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
Add a Townhouse Outreach tab for townhouse developers and volume builders
A separate message for the three approved and raw townhouse sites in
Tarneit, Weir Views, Werribee and Geelong, addressed to the 29 townhouse
developers and builder/developers already in the list. Volume builders
found by further research are added from build/builders.json when present.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -9,16 +9,18 @@
   <sheets>
     <sheet name="Developer List" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Outreach" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cross-check" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="UDIA All Members" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sources &amp; Notes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Townhouse Outreach" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cross-check" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="UDIA All Members" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Sources &amp; Notes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Developer List'!$A$1:$V$197</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Outreach'!$A$1:$N$195</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Cross-check'!$A$1:$B$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'UDIA All Members'!$A$1:$H$386</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sources &amp; Notes'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Townhouse Outreach'!$A$1:$I$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cross-check'!$A$1:$B$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'UDIA All Members'!$A$1:$H$386</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sources &amp; Notes'!$A$1:$B$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32499,6 +32501,1808 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Developer / builder</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Phone</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Message</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="300" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Metricon Homes</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>customerservice@metricon.com.au</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>03 9915 5555</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>https://www.metricon.com.au/</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Metricon's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3" ht="300" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Carlisle Homes</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>customerenquiry@carlislehomes.com.au</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>03 8108 3630</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>https://www.carlislehomes.com.au/</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Carlisle Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="300" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Simonds Homes Victoria</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>customer.success@simonds.com.au</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>03 9682 0700</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>https://www.simonds.com.au/</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Simonds' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5" ht="300" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Burbank Group</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>build@burbank.com.au</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>13 28 72</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>https://www.burbank.com.au/</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Burbank's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="300" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Glenvill Homes</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>enquiry@glenvill.com.au</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>03 9573 8393</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>https://glenvill.com.au/</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Glenvill Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="300" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SJD Homes</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>info@sjdhomes.com.au</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>03 5940 4206</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sjdhomes.com.au/</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SJD Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="300" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Creation Homes</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>info@creationhomes.com.au</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>03 9828 0700</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.creationhomes.com.au/</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Creation Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="300" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Hudson Ridge Builders</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>hello@hudsonridge.com.au</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>03 5332 6889</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Hudson Ridge Builders' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="300" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Integra Group</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@integragroup.com.au</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>03 5322 5999</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.integragroup.com.au</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Integra Group's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="300" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Kode Living</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>sales@kodeliving.com.au</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>0499 883 888</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Kode Living's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="300" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Mirvac</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>viccustomer@mirvac.com</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>+61 3 9695 9400</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mirvac.com</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Mirvac's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="300" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SOHO Living</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>info@soholiving.com.au</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>13 76 46</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.soholiving.com.au</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SOHO Living's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="300" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Oreana</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>info@oreana.com.au</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>+61 3 9804 7113</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>https://oreana.com.au</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Oreana's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="300" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Arc Living</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>hello@arcliving.com.au</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>1300 877 767</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>https://arcliving.com.au</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Arc Living's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="300" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Hub Property Group</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>info@hubpg.com.au</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>03 9081 1611</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Hub Property Group's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="300" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Hygge Property</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>hello@hyggeproperty.com.au</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Hygge Property's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="300" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Little Projects</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>info@littleprojects.com.au</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>https://littleprojects.com.au/</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Little Projects' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="300" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Lowe Living</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>info@loweliving.com.au</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>03 9598 7357</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>https://loweliving.com.au/</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Lowe Living's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="300" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Maax Global</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>info@maaxglobal.com.au</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>03 9117 5425</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Maax Global's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="300" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>OYOB Property Group</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>info@oyob.com.au</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>03 9818 1467</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oyob.com.au</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit OYOB Property Group's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="300" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Resimax Group</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>info@resimaxgroup.com.au</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>1300 858 190</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>https://www.resimaxgroup.com.au/</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Resimax Group's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="300" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Resi Ventures</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>land@resiventures.com.au</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>1300 031 260</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>https://resiventures.com.au/</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Resi Ventures' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="300" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>SIG Group</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>admin@siggroup.com.au</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>03 9998 2408</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>https://siggroup.com.au</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SIG Group's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="300" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>SightStone</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>admin@sightstone.com</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>03 9098 0712</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sightstone.com/</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SightStone's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="300" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>SYP Property</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>info@syproperty.com</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>03 9600 0590</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>https://syproperty.com/</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SYP Property's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="300" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Sunkin Property Group</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>office@sunkin.com.au</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>13 68 88</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>https://sunkin.com.au/</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Sunkin Property Group's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="300" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Milieu</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>info@milieuproperty.com.au</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>03 9699 5000</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>https://milieu.com.au/</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Milieu's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29" ht="300" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ID_Land</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>info@idland.com.au</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>+61 3 9867 4700</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>https://idland.com.au</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit ID_Land's townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="300" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Antipodean Land Developments</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>vali.valibhoy@gmail.com</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Developer list</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Antipodean Land Developments' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I30"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId23"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -32764,7 +34568,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47024,7 +48828,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add volume builders to the Townhouse Outreach tab
Orbit, Sherridon, Boutique, JG King, Fairhaven, Mimosa and Eight Homes
join the townhouse campaign from build/builders.json. Henley publishes no
enquiries email, Rawdon Hill is in liquidation, Dennis Family Homes now
sits under Simonds, and the only Hallmark Homes found is in Queensland, so
none of those four are emailed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -17,7 +17,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Developer List'!$A$1:$V$197</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Outreach'!$A$1:$N$195</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Townhouse Outreach'!$A$1:$I$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Townhouse Outreach'!$A$1:$I$37</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cross-check'!$A$1:$B$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'UDIA All Members'!$A$1:$H$386</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Sources &amp; Notes'!$A$1:$B$11</definedName>
@@ -32501,7 +32501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -34266,8 +34266,456 @@
       </c>
       <c r="I30" s="3" t="inlineStr"/>
     </row>
+    <row r="31" ht="300" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Orbit Homes</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>info@orbithomes.com.au</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>03 9377 0000</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>https://orbithomes.com.au</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Volume builder research</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Orbit Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Email published on official LinkedIn page; privacy policy also points to info@orbithomes.com... (truncated excerpt). Contact page has form only. VIC head office: 286 Mt Alexander Rd, Ascot Vale VIC 3032; sales line 1300 672 484.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="300" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Sherridon Homes</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>info@sherridonhomes.com.au</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>1300 188 668</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sherridonhomes.com.au</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>Volume builder research</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Sherridon Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Email seen only on a golf club sponsor post, not an official Sherridon page. Company website has contact form only. Email comes from a third-party sponsor post (Traralgon Golf Club Facebook) that lists Sherridon's details, not from an official Sherridon page, so verify before relying on it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="300" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Boutique Homes</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@boutiquehomes.com.au</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>03 9674 4500</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.boutiquehomes.com.au</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Volume builder research</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Boutique Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Email from official Facebook page. Part of ABN Group. Website contact page lists only the warranty email warranty@abngroup.com.au / (03) 9674 4554. HQ Docklands VIC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="300" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>JG King Homes</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>marketing@jgking.com.au</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>1300 545 464</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>https://jgkinghomes.com.au</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>Volume builder research</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit JG King Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Marketing email from official Facebook contact info; no general or land email seen. Website contact page has form only. HQ Port Melbourne VIC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="300" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Fairhaven Homes</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>info@fairhavenhomes.com.au</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>1800 324 742</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>https://fairhavenhomes.com.au</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Volume builder research</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Fairhaven Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>1800 Fairhaven; sales 0400 660 960. Level 6, 1 Peters Ave, Mulgrave VIC 3170.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="300" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Mimosa Homes</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>info@mimosahomes.com.au</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>(03) 8361 1900</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mimosahomes.com.au</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>Volume builder research</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Mimosa Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Head office email. Also 1300 MIMOSA (1300 646 672); sales@mimosahomes.com.au is listed on the head-office display page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="300" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Eight Homes</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>enquiry@8homes.com.au</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>(03) 8398 1000</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.8homes.com.au</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Volume builder research</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Townhouse sites – Tarneit, Weir Views, Werribee &amp; Geelong</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Hi Acquisition team,
+Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Eight Homes' townhouse pipeline:
+* Permit-approved townhouse sites for a faster start.
+* Raw townhouse sites with room to design your own scheme.
+* Central locations in Tarneit, Weir Views, Werribee and Geelong.
+Who in acquisitions should I send the details to?
+If it's not a fit, just let me know and I won't follow up.
+Kind Regards,
+Inder Sandhu
+Principal /OIEC
+CROWN REAL ESTATE AGENTS
+Phone no: 0484 926 324
+Inder@crownrea.com.au
+Disclaimer : This email and any attachments are confidential and intended solely for the intended recipient(s). If you are not the intended recipient, please notify the sender immediately, delete this email, and refrain from disclosing, copying, or using any part of this communication.
+The information in this email is for general informational purposes only and should not be considered legal, financial, or professional advice. Crown Real Estate Agencts makes no guarantees regarding its accuracy or completeness. Any views expressed are those of the author and do not necessarily reflect the views of Crown Real Estate Agents.
+Crown Real Estate Agents complies with all relevant Victorian and Australian laws, including the Estate Agents Act 1980 (Vic) and the Australian Consumer Law. We are committed to fair trading, privacy, and anti-discrimination practices, as required by the Equal Opportunity Act 2010 (Vic) and the Privacy Act 1988 (Cth).
+While precautions are taken to prevent viruses, Crown Real Estate Agents accepts no liability for damage caused by email transmission.
+No binding agreements may be concluded via email without written confirmation by an authorised representative of Crown Real Estate Agents.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Also shown in the privacy policy. Sales line 03 8398 1188.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I30"/>
+  <autoFilter ref="A1:I37"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -34292,6 +34740,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId30"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Mark the 36 townhouse drafts on the Townhouse Outreach tab
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -32617,7 +32617,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr"/>
@@ -32677,7 +32677,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr"/>
@@ -32737,7 +32737,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr"/>
@@ -32797,7 +32797,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr"/>
@@ -32857,7 +32857,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr"/>
@@ -32917,7 +32917,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr"/>
@@ -32977,7 +32977,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr"/>
@@ -33033,7 +33033,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr"/>
@@ -33093,7 +33093,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr"/>
@@ -33149,7 +33149,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr"/>
@@ -33209,7 +33209,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr"/>
@@ -33269,7 +33269,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr"/>
@@ -33329,7 +33329,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr"/>
@@ -33389,7 +33389,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr"/>
@@ -33445,7 +33445,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr"/>
@@ -33497,7 +33497,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr"/>
@@ -33553,7 +33553,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr"/>
@@ -33613,7 +33613,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr"/>
@@ -33669,7 +33669,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr"/>
@@ -33729,7 +33729,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr"/>
@@ -33789,7 +33789,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr"/>
@@ -33849,7 +33849,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr"/>
@@ -33909,7 +33909,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr"/>
@@ -33969,7 +33969,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr"/>
@@ -34029,7 +34029,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr"/>
@@ -34089,7 +34089,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr"/>
@@ -34149,7 +34149,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr"/>
@@ -34209,7 +34209,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr"/>
@@ -34261,7 +34261,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr"/>
@@ -34321,7 +34321,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -34385,7 +34385,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -34449,7 +34449,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -34513,7 +34513,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -34577,7 +34577,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -34641,7 +34641,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -34705,7 +34705,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Not sent</t>
+          <t>Draft created 2026-10-03</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Townhouse email: four sites, not three
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -32596,7 +32596,7 @@
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Metricon's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Metricon's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -32656,7 +32656,7 @@
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Carlisle Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Carlisle Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -32716,7 +32716,7 @@
       <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Simonds' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Simonds' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -32776,7 +32776,7 @@
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Burbank's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Burbank's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -32836,7 +32836,7 @@
       <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Glenvill Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Glenvill Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -32896,7 +32896,7 @@
       <c r="G7" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SJD Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SJD Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -32956,7 +32956,7 @@
       <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Creation Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Creation Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33012,7 +33012,7 @@
       <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Hudson Ridge Builders' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Hudson Ridge Builders' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33072,7 +33072,7 @@
       <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Integra Group's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Integra Group's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33128,7 +33128,7 @@
       <c r="G11" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Kode Living's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Kode Living's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33188,7 +33188,7 @@
       <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Mirvac's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Mirvac's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33248,7 +33248,7 @@
       <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SOHO Living's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SOHO Living's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33308,7 +33308,7 @@
       <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Oreana's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Oreana's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33368,7 +33368,7 @@
       <c r="G15" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Arc Living's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Arc Living's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33424,7 +33424,7 @@
       <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Hub Property Group's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Hub Property Group's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33476,7 +33476,7 @@
       <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Hygge Property's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Hygge Property's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33532,7 +33532,7 @@
       <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Little Projects' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Little Projects' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33592,7 +33592,7 @@
       <c r="G19" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Lowe Living's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Lowe Living's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33648,7 +33648,7 @@
       <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Maax Global's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Maax Global's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33708,7 +33708,7 @@
       <c r="G21" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit OYOB Property Group's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit OYOB Property Group's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33768,7 +33768,7 @@
       <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Resimax Group's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Resimax Group's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33828,7 +33828,7 @@
       <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Resi Ventures' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Resi Ventures' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33888,7 +33888,7 @@
       <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SIG Group's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SIG Group's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -33948,7 +33948,7 @@
       <c r="G25" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SightStone's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SightStone's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34008,7 +34008,7 @@
       <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SYP Property's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit SYP Property's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34068,7 +34068,7 @@
       <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Sunkin Property Group's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Sunkin Property Group's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34128,7 +34128,7 @@
       <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Milieu's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Milieu's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34188,7 +34188,7 @@
       <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit ID_Land's townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit ID_Land's townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34240,7 +34240,7 @@
       <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Antipodean Land Developments' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Antipodean Land Developments' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34300,7 +34300,7 @@
       <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Orbit Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Orbit Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34364,7 +34364,7 @@
       <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Sherridon Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Sherridon Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34428,7 +34428,7 @@
       <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Boutique Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Boutique Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34492,7 +34492,7 @@
       <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit JG King Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit JG King Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34556,7 +34556,7 @@
       <c r="G35" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Fairhaven Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Fairhaven Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34620,7 +34620,7 @@
       <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Mimosa Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Mimosa Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.
@@ -34684,7 +34684,7 @@
       <c r="G37" s="3" t="inlineStr">
         <is>
           <t>Hi Acquisition team,
-Quick one. I'm representing three townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Eight Homes' townhouse pipeline:
+Quick one. I'm representing four townhouse sites, both permit-approved and raw, in the heart of Tarneit, Weir Views, Werribee and Geelong that could suit Eight Homes' townhouse pipeline:
 * Permit-approved townhouse sites for a faster start.
 * Raw townhouse sites with room to design your own scheme.
 * Central locations in Tarneit, Weir Views, Werribee and Geelong.

</xml_diff>

<commit_message>
Mark Creation Homes and Lowe Living townhouse emails as sent
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -32977,7 +32977,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-03 (by Inder)</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr"/>
@@ -33613,7 +33613,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-03 (by Inder)</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Mark the townhouse campaign as sent
32 townhouse emails sent from their drafts on 4 October; Simonds, Burbank,
Creation Homes and Lowe Living were sent by hand.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014BGBs4NHeym6Czgaf1SqKJ
</commit_message>
<xml_diff>
--- a/prospecting/developer_list/Victorian_Developer_List.xlsx
+++ b/prospecting/developer_list/Victorian_Developer_List.xlsx
@@ -32617,7 +32617,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr"/>
@@ -32677,7 +32677,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr"/>
@@ -32737,7 +32737,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04 (by Inder)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr"/>
@@ -32797,7 +32797,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04 (by Inder)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr"/>
@@ -32857,7 +32857,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr"/>
@@ -32917,7 +32917,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr"/>
@@ -33033,7 +33033,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr"/>
@@ -33093,7 +33093,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr"/>
@@ -33149,7 +33149,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr"/>
@@ -33209,7 +33209,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr"/>
@@ -33269,7 +33269,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr"/>
@@ -33329,7 +33329,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr"/>
@@ -33389,7 +33389,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr"/>
@@ -33445,7 +33445,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr"/>
@@ -33497,7 +33497,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr"/>
@@ -33553,7 +33553,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr"/>
@@ -33669,7 +33669,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr"/>
@@ -33729,7 +33729,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr"/>
@@ -33789,7 +33789,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr"/>
@@ -33849,7 +33849,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr"/>
@@ -33909,7 +33909,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr"/>
@@ -33969,7 +33969,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr"/>
@@ -34029,7 +34029,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr"/>
@@ -34089,7 +34089,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr"/>
@@ -34149,7 +34149,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr"/>
@@ -34209,7 +34209,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr"/>
@@ -34261,7 +34261,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr"/>
@@ -34321,7 +34321,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
@@ -34385,7 +34385,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
@@ -34449,7 +34449,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
@@ -34513,7 +34513,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -34577,7 +34577,7 @@
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -34641,7 +34641,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
@@ -34705,7 +34705,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Draft created 2026-10-03</t>
+          <t>Sent 2026-10-04</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">

</xml_diff>